<commit_message>
Linking settings tab to selection tab
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B555BB6E-6CFF-4373-B488-29A0AD85B418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1404BA23-D8A2-4886-9752-EF7DD002CCC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="exiobase" sheetId="1" r:id="rId1"/>
-    <sheet name="german" sheetId="2" r:id="rId2"/>
-    <sheet name="english" sheetId="3" r:id="rId3"/>
+    <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
+    <sheet name="Deutsch" sheetId="2" r:id="rId2"/>
+    <sheet name="English" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>

<commit_message>
Added general dict to ui
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1404BA23-D8A2-4886-9752-EF7DD002CCC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2484CCB7-B1EC-4D70-A574-07D48C5C7222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="40">
   <si>
     <t>exiobase</t>
   </si>
@@ -104,6 +104,48 @@
   <si>
     <t>Rohstoff-
 gewinnung</t>
+  </si>
+  <si>
+    <t>Selection</t>
+  </si>
+  <si>
+    <t>Auswahl</t>
+  </si>
+  <si>
+    <t>Visualisation</t>
+  </si>
+  <si>
+    <t>Settings</t>
+  </si>
+  <si>
+    <t>Visualisierung</t>
+  </si>
+  <si>
+    <t>Einstellungen</t>
+  </si>
+  <si>
+    <t>General Settings</t>
+  </si>
+  <si>
+    <t>Grundeinstellungen</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Sprache</t>
+  </si>
+  <si>
+    <t>Jahr</t>
+  </si>
+  <si>
+    <t>Show Indices</t>
+  </si>
+  <si>
+    <t>Indices anzeigen</t>
   </si>
 </sst>
 </file>
@@ -147,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -170,11 +212,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -186,6 +239,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -488,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -590,6 +644,62 @@
         <v>20</v>
       </c>
     </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -597,7 +707,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" customWidth="1"/>
@@ -700,6 +810,62 @@
         <v>15</v>
       </c>
     </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -707,7 +873,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -810,6 +976,94 @@
         <v>21</v>
       </c>
     </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added full translation to all tabs and config data
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2484CCB7-B1EC-4D70-A574-07D48C5C7222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D9E3B48-4A10-4F15-9965-96681AA17653}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="84">
   <si>
     <t>exiobase</t>
   </si>
@@ -146,6 +146,138 @@
   </si>
   <si>
     <t>Indices anzeigen</t>
+  </si>
+  <si>
+    <t>Region Selection</t>
+  </si>
+  <si>
+    <t>Region-Auswahl</t>
+  </si>
+  <si>
+    <t>Clear</t>
+  </si>
+  <si>
+    <t>Lösche</t>
+  </si>
+  <si>
+    <t>Select All Regions</t>
+  </si>
+  <si>
+    <t>Wähle alle Regionen aus</t>
+  </si>
+  <si>
+    <t>Sector Selection</t>
+  </si>
+  <si>
+    <t>Select All Sectors</t>
+  </si>
+  <si>
+    <t>Sektor-Auswahl</t>
+  </si>
+  <si>
+    <t>Wähle alle Sektoren aus</t>
+  </si>
+  <si>
+    <t>Selection Summary</t>
+  </si>
+  <si>
+    <t>Zusammenfassung der Auswahl</t>
+  </si>
+  <si>
+    <t>No selection made</t>
+  </si>
+  <si>
+    <t>Keine Auswahl getroffen</t>
+  </si>
+  <si>
+    <t>Apply Selection</t>
+  </si>
+  <si>
+    <t>Aktuelle Auswahl übernehmen</t>
+  </si>
+  <si>
+    <t>Reset All Selections</t>
+  </si>
+  <si>
+    <t>Alles zurücksetzen</t>
+  </si>
+  <si>
+    <t>Regions</t>
+  </si>
+  <si>
+    <t>Regionen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sectors </t>
+  </si>
+  <si>
+    <t>Sektoren</t>
+  </si>
+  <si>
+    <t>No regions selected</t>
+  </si>
+  <si>
+    <t>No sectors selected</t>
+  </si>
+  <si>
+    <t>Keine Regionen ausgewählt</t>
+  </si>
+  <si>
+    <t>Keine Sektoren ausgewählt</t>
+  </si>
+  <si>
+    <t>All regions selected (Global view)</t>
+  </si>
+  <si>
+    <t>All sectors selected (Global view)</t>
+  </si>
+  <si>
+    <t>Alle Regionen ausgewählt (Globale Ansicht)</t>
+  </si>
+  <si>
+    <t>Alle Sektoren ausgewählt (Globale Ansicht)</t>
+  </si>
+  <si>
+    <t>Sector indices count</t>
+  </si>
+  <si>
+    <t>Anzahl der Sektoren</t>
+  </si>
+  <si>
+    <t>Region indices count</t>
+  </si>
+  <si>
+    <t>Anzahl der Regionen</t>
+  </si>
+  <si>
+    <t>World Map</t>
+  </si>
+  <si>
+    <t>Weltkarte</t>
+  </si>
+  <si>
+    <t>Select Impacts</t>
+  </si>
+  <si>
+    <t>Wähle Umweltindikatoren</t>
+  </si>
+  <si>
+    <t>Selected</t>
+  </si>
+  <si>
+    <t>Ausgewählt</t>
+  </si>
+  <si>
+    <t>Update Plot</t>
+  </si>
+  <si>
+    <t>Plot aktualisieren</t>
+  </si>
+  <si>
+    <t>Reset to Defaults</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zurücksetzen </t>
   </si>
 </sst>
 </file>
@@ -227,7 +359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -239,7 +371,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -542,10 +675,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="31.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -645,59 +778,235 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -707,11 +1016,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" customWidth="1"/>
-    <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -798,7 +1107,7 @@
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -811,73 +1120,249 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="2" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="31.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -977,91 +1462,267 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="A21" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="A22" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added title to supply chain analysis
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA837A77-4C53-49D4-BEF2-ADE63D3E2BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B0A9C63-810D-419F-9365-F91D93A0B7CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="88">
   <si>
     <t>exiobase</t>
   </si>
@@ -278,6 +278,18 @@
   </si>
   <si>
     <t>Sectors</t>
+  </si>
+  <si>
+    <t>of a</t>
+  </si>
+  <si>
+    <t>einer</t>
+  </si>
+  <si>
+    <t>spezifischen Auswahl von Sektoren</t>
+  </si>
+  <si>
+    <t>specific selection of sectors</t>
   </si>
 </sst>
 </file>
@@ -359,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -372,6 +384,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -674,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="31.140625" bestFit="1" customWidth="1"/>
@@ -1008,6 +1021,22 @@
         <v>81</v>
       </c>
     </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1015,7 +1044,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.140625" bestFit="1" customWidth="1"/>
@@ -1350,6 +1379,22 @@
         <v>82</v>
       </c>
     </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1358,7 +1403,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="31.140625" bestFit="1" customWidth="1"/>
@@ -1724,6 +1769,22 @@
         <v>81</v>
       </c>
     </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed language switch for the settings tab
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F100EDE7-C73E-43CE-A4B7-6CC523F10940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{271EFA71-72EC-4AEC-8E71-98DABE6CB7D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="93">
   <si>
     <t>exiobase</t>
   </si>
@@ -302,6 +302,9 @@
   </si>
   <si>
     <t>world</t>
+  </si>
+  <si>
+    <t>Optionen</t>
   </si>
 </sst>
 </file>
@@ -2109,7 +2112,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="38.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="46.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="9.140625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -2603,7 +2606,7 @@
         <v>46</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>60</v>
+        <v>92</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45" s="5"/>

</xml_diff>

<commit_message>
New impact matrices, divided in regional impacts
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17308410-2E67-4E5F-8BEC-2A8644A87513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{723CC9E3-D999-48CF-886D-7C531E4D789C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="105">
   <si>
     <t>exiobase</t>
   </si>
@@ -335,6 +335,12 @@
   </si>
   <si>
     <t>mehr Input benötigt</t>
+  </si>
+  <si>
+    <t>Global</t>
+  </si>
+  <si>
+    <t>Globale/r/s</t>
   </si>
 </sst>
 </file>
@@ -380,7 +386,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -390,46 +396,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="12"/>
-      </right>
-      <top style="thin">
-        <color indexed="12"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="12"/>
-      </left>
-      <right style="thin">
-        <color indexed="12"/>
-      </right>
-      <top style="thin">
-        <color indexed="12"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -437,18 +413,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1612,559 +1587,429 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="38.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="38.42578125" style="4" customWidth="1"/>
     <col min="3" max="6" width="9.140625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+    </row>
+    <row r="2" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-    </row>
-    <row r="4" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    </row>
+    <row r="4" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-    </row>
-    <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    </row>
+    <row r="5" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-    </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+    </row>
+    <row r="6" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-    </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+    </row>
+    <row r="9" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+    </row>
+    <row r="10" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    </row>
+    <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+    </row>
+    <row r="13" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+    </row>
+    <row r="14" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-    </row>
-    <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+    </row>
+    <row r="15" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-    </row>
-    <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+    </row>
+    <row r="16" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-    </row>
-    <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+    </row>
+    <row r="17" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-    </row>
-    <row r="18" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+    </row>
+    <row r="18" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-    </row>
-    <row r="19" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+    </row>
+    <row r="19" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-    </row>
-    <row r="20" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+    </row>
+    <row r="20" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-    </row>
-    <row r="21" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+    </row>
+    <row r="21" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-    </row>
-    <row r="22" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+    </row>
+    <row r="22" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-    </row>
-    <row r="23" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+    </row>
+    <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-    </row>
-    <row r="24" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+    </row>
+    <row r="24" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="4"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-    </row>
-    <row r="25" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+    </row>
+    <row r="25" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-    </row>
-    <row r="26" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
+    </row>
+    <row r="26" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-    </row>
-    <row r="27" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
+    </row>
+    <row r="27" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-    </row>
-    <row r="28" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
+    </row>
+    <row r="28" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-    </row>
-    <row r="29" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+    </row>
+    <row r="29" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C29" s="4"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-    </row>
-    <row r="30" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+    </row>
+    <row r="30" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-    </row>
-    <row r="31" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+    </row>
+    <row r="31" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-    </row>
-    <row r="32" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
+    </row>
+    <row r="32" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C32" s="4"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-    </row>
-    <row r="33" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
+    </row>
+    <row r="33" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C33" s="4"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-    </row>
-    <row r="34" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
+    </row>
+    <row r="34" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C34" s="4"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-    </row>
-    <row r="35" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
+    </row>
+    <row r="35" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-    </row>
-    <row r="36" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
+    </row>
+    <row r="36" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-    </row>
-    <row r="37" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
+    </row>
+    <row r="37" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-    </row>
-    <row r="38" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
+    </row>
+    <row r="38" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-    </row>
-    <row r="39" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
+    </row>
+    <row r="39" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C39" s="4"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
-    </row>
-    <row r="40" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="6" t="s">
+    </row>
+    <row r="40" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C40" s="4"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-    </row>
-    <row r="41" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
+    </row>
+    <row r="41" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C41" s="4"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-    </row>
-    <row r="42" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="6" t="s">
+    </row>
+    <row r="42" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C42" s="4"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-    </row>
-    <row r="43" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
+    </row>
+    <row r="43" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C43" s="4"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-    </row>
-    <row r="44" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
+    </row>
+    <row r="44" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C44" s="4"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-    </row>
-    <row r="45" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
+    </row>
+    <row r="45" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C45" s="4"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-    </row>
-    <row r="46" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="6" t="s">
+    </row>
+    <row r="46" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-    </row>
-    <row r="47" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="6" t="s">
+    </row>
+    <row r="47" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="6" t="s">
+    <row r="48" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="2" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
+      <c r="A49" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="2" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="2" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="6" t="s">
+      <c r="A51" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="2" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2178,559 +2023,429 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="46.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="46.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="9.140625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+    </row>
+    <row r="2" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-    </row>
-    <row r="4" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    </row>
+    <row r="4" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-    </row>
-    <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    </row>
+    <row r="5" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-    </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+    </row>
+    <row r="6" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-    </row>
-    <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+    </row>
+    <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+    </row>
+    <row r="10" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    </row>
+    <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+    </row>
+    <row r="13" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+    </row>
+    <row r="14" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-    </row>
-    <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+    </row>
+    <row r="15" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-    </row>
-    <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+    </row>
+    <row r="16" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-    </row>
-    <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+    </row>
+    <row r="17" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-    </row>
-    <row r="18" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+    </row>
+    <row r="18" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-    </row>
-    <row r="19" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+    </row>
+    <row r="19" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-    </row>
-    <row r="20" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+    </row>
+    <row r="20" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-    </row>
-    <row r="21" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+    </row>
+    <row r="21" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-    </row>
-    <row r="22" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+    </row>
+    <row r="22" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-    </row>
-    <row r="23" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+    </row>
+    <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-    </row>
-    <row r="24" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+    </row>
+    <row r="24" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C24" s="4"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-    </row>
-    <row r="25" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+    </row>
+    <row r="25" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-    </row>
-    <row r="26" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
+    </row>
+    <row r="26" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-    </row>
-    <row r="27" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
+    </row>
+    <row r="27" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-    </row>
-    <row r="28" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
+    </row>
+    <row r="28" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-    </row>
-    <row r="29" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+    </row>
+    <row r="29" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C29" s="4"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-    </row>
-    <row r="30" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+    </row>
+    <row r="30" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-    </row>
-    <row r="31" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+    </row>
+    <row r="31" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-    </row>
-    <row r="32" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
+    </row>
+    <row r="32" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C32" s="4"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-    </row>
-    <row r="33" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
+    </row>
+    <row r="33" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="4"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-    </row>
-    <row r="34" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
+    </row>
+    <row r="34" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C34" s="4"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-    </row>
-    <row r="35" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
+    </row>
+    <row r="35" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-    </row>
-    <row r="36" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
+    </row>
+    <row r="36" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-    </row>
-    <row r="37" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
+    </row>
+    <row r="37" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-    </row>
-    <row r="38" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
+    </row>
+    <row r="38" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-    </row>
-    <row r="39" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
+    </row>
+    <row r="39" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C39" s="4"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
-    </row>
-    <row r="40" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="6" t="s">
+    </row>
+    <row r="40" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C40" s="4"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-    </row>
-    <row r="41" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
+    </row>
+    <row r="41" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C41" s="4"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-    </row>
-    <row r="42" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="6" t="s">
+    </row>
+    <row r="42" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C42" s="4"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-    </row>
-    <row r="43" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
+    </row>
+    <row r="43" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C43" s="4"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-    </row>
-    <row r="44" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
+    </row>
+    <row r="44" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C44" s="4"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-    </row>
-    <row r="45" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
+    </row>
+    <row r="45" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C45" s="4"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-    </row>
-    <row r="46" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="6" t="s">
+    </row>
+    <row r="46" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-    </row>
-    <row r="47" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="6" t="s">
+    </row>
+    <row r="47" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="6" t="s">
+    <row r="48" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="2" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
+      <c r="A49" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="2" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="2" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="6" t="s">
+      <c r="A51" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="2" t="s">
         <v>102</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2744,603 +2459,461 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="38.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="38.42578125" style="4" customWidth="1"/>
     <col min="3" max="6" width="9.140625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+    </row>
+    <row r="2" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-    </row>
-    <row r="4" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    </row>
+    <row r="4" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-    </row>
-    <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    </row>
+    <row r="5" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-    </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+    </row>
+    <row r="6" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-    </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+    </row>
+    <row r="9" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+    </row>
+    <row r="10" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    </row>
+    <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+    </row>
+    <row r="13" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+    </row>
+    <row r="14" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-    </row>
-    <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+    </row>
+    <row r="15" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-    </row>
-    <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+    </row>
+    <row r="16" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-    </row>
-    <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+    </row>
+    <row r="17" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-    </row>
-    <row r="18" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+    </row>
+    <row r="18" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-    </row>
-    <row r="19" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+    </row>
+    <row r="19" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-    </row>
-    <row r="20" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+    </row>
+    <row r="20" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-    </row>
-    <row r="21" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+    </row>
+    <row r="21" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-    </row>
-    <row r="22" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+    </row>
+    <row r="22" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-    </row>
-    <row r="23" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+    </row>
+    <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-    </row>
-    <row r="24" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+    </row>
+    <row r="24" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="4"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-    </row>
-    <row r="25" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+    </row>
+    <row r="25" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-    </row>
-    <row r="26" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
+    </row>
+    <row r="26" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-    </row>
-    <row r="27" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
+    </row>
+    <row r="27" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-    </row>
-    <row r="28" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
+    </row>
+    <row r="28" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-    </row>
-    <row r="29" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+    </row>
+    <row r="29" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C29" s="4"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-    </row>
-    <row r="30" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+    </row>
+    <row r="30" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-    </row>
-    <row r="31" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+    </row>
+    <row r="31" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-    </row>
-    <row r="32" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
+    </row>
+    <row r="32" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C32" s="4"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-    </row>
-    <row r="33" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
+    </row>
+    <row r="33" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C33" s="4"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-    </row>
-    <row r="34" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
+    </row>
+    <row r="34" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="4"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-    </row>
-    <row r="35" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
+    </row>
+    <row r="35" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-    </row>
-    <row r="36" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
+    </row>
+    <row r="36" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-    </row>
-    <row r="37" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
+    </row>
+    <row r="37" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-    </row>
-    <row r="38" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
+    </row>
+    <row r="38" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-    </row>
-    <row r="39" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
+    </row>
+    <row r="39" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C39" s="4"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
-    </row>
-    <row r="40" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="6" t="s">
+    </row>
+    <row r="40" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C40" s="4"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-    </row>
-    <row r="41" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
+    </row>
+    <row r="41" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C41" s="4"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-    </row>
-    <row r="42" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="6" t="s">
+    </row>
+    <row r="42" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C42" s="4"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-    </row>
-    <row r="43" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
+    </row>
+    <row r="43" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C43" s="4"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-    </row>
-    <row r="44" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
+    </row>
+    <row r="44" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="4"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-    </row>
-    <row r="45" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
+    </row>
+    <row r="45" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="4"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-    </row>
-    <row r="46" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="6" t="s">
+    </row>
+    <row r="46" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-    </row>
-    <row r="47" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="6" t="s">
+    </row>
+    <row r="47" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C47" s="4"/>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
-    </row>
-    <row r="48" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="6" t="s">
+    </row>
+    <row r="48" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C48" s="4"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-    </row>
-    <row r="49" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
+    </row>
+    <row r="49" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C49" s="4"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-    </row>
-    <row r="50" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="6" t="s">
+    </row>
+    <row r="50" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C50" s="4"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
-    </row>
-    <row r="51" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="6" t="s">
+    </row>
+    <row r="51" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="6" t="s">
+    <row r="52" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="6" t="s">
+    <row r="53" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="B53" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="6" t="s">
+    <row r="54" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="6" t="s">
+    <row r="55" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B55" s="6" t="s">
+      <c r="B55" s="2" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Minor Changes to general.xlsx (translations)
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05A089F5-E02F-424B-94F4-4CB0E893B7E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4725C90C-6A53-4ED4-8F94-7228F83DCF55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="111">
   <si>
     <t>exiobase</t>
   </si>
@@ -353,6 +353,12 @@
   </si>
   <si>
     <t>Bitte aktualisieren</t>
+  </si>
+  <si>
+    <t>of the World</t>
+  </si>
+  <si>
+    <t>der Welt</t>
   </si>
 </sst>
 </file>
@@ -1606,7 +1612,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -2047,6 +2053,14 @@
         <v>107</v>
       </c>
     </row>
+    <row r="55" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
@@ -2058,7 +2072,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -2499,6 +2513,14 @@
         <v>108</v>
       </c>
     </row>
+    <row r="55" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
@@ -2510,7 +2532,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -2983,6 +3005,14 @@
         <v>107</v>
       </c>
     </row>
+    <row r="59" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Minor design changes to the ToolTip Dialog
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11678D8E-9851-4A40-90D9-C507DEC13C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2D29FAC-731B-4E6C-85DA-838427FF63F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="121">
   <si>
     <t>exiobase</t>
   </si>
@@ -377,6 +377,18 @@
   </si>
   <si>
     <t>Plot abspeichern</t>
+  </si>
+  <si>
+    <t>Percentage</t>
+  </si>
+  <si>
+    <t>Prozentwert</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Info</t>
   </si>
 </sst>
 </file>
@@ -1630,7 +1642,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -2103,6 +2115,30 @@
         <v>114</v>
       </c>
     </row>
+    <row r="59" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
@@ -2114,7 +2150,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -2587,6 +2623,30 @@
         <v>115</v>
       </c>
     </row>
+    <row r="59" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
@@ -2598,7 +2658,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B62"/>
+  <dimension ref="A1:B65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -3103,6 +3163,30 @@
         <v>114</v>
       </c>
     </row>
+    <row r="63" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
New plot worldmap function
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{296C6D6A-3466-4163-976C-5BEDE8FC27B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CECBB5E2-663F-4FB1-8F35-A0D3063AA90F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -177,9 +177,6 @@
     <t>Farbe</t>
   </si>
   <si>
-    <t>Einzelhandel</t>
-  </si>
-  <si>
     <t>Direkte
 Zulieferer</t>
   </si>
@@ -431,6 +428,10 @@
   </si>
   <si>
     <t>Dunkelmodus</t>
+  </si>
+  <si>
+    <t>Konsumgüter-
+produktion</t>
   </si>
 </sst>
 </file>
@@ -2075,130 +2076,130 @@
     </row>
     <row r="47" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C62" s="8"/>
       <c r="D62" s="8"/>
@@ -2211,50 +2212,50 @@
     </row>
     <row r="63" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="64" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -2317,12 +2318,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>51</v>
+      <c r="B6" s="6" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2330,7 +2331,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2338,7 +2339,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2346,7 +2347,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2354,7 +2355,7 @@
         <v>11</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2362,7 +2363,7 @@
         <v>12</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2370,7 +2371,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2378,7 +2379,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2386,7 +2387,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2394,7 +2395,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2402,7 +2403,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2410,7 +2411,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2418,7 +2419,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2426,7 +2427,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2434,7 +2435,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2442,7 +2443,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2450,7 +2451,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2458,7 +2459,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2466,7 +2467,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2474,7 +2475,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2482,7 +2483,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2490,7 +2491,7 @@
         <v>27</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2498,7 +2499,7 @@
         <v>28</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2506,7 +2507,7 @@
         <v>29</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2514,7 +2515,7 @@
         <v>30</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2522,7 +2523,7 @@
         <v>31</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2530,7 +2531,7 @@
         <v>32</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2538,7 +2539,7 @@
         <v>33</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2546,7 +2547,7 @@
         <v>34</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2554,7 +2555,7 @@
         <v>35</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2562,7 +2563,7 @@
         <v>36</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2570,7 +2571,7 @@
         <v>37</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2578,7 +2579,7 @@
         <v>38</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2586,7 +2587,7 @@
         <v>39</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2594,7 +2595,7 @@
         <v>40</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2602,7 +2603,7 @@
         <v>41</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2610,7 +2611,7 @@
         <v>42</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2618,7 +2619,7 @@
         <v>43</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2634,7 +2635,7 @@
         <v>46</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2642,183 +2643,183 @@
         <v>19</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B52" s="4" t="s">
         <v>103</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B54" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="B54" s="7" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B55" s="4" t="s">
         <v>109</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B56" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B58" s="7" t="s">
         <v>114</v>
-      </c>
-      <c r="B58" s="7" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B59" s="7" t="s">
         <v>119</v>
-      </c>
-      <c r="B59" s="7" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B62" s="4" t="s">
         <v>121</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B63" s="7" t="s">
         <v>123</v>
-      </c>
-      <c r="B63" s="7" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B64" s="7" t="s">
         <v>125</v>
-      </c>
-      <c r="B64" s="7" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B65" t="s">
         <v>127</v>
-      </c>
-      <c r="B65" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B67" s="7" t="s">
         <v>131</v>
-      </c>
-      <c r="B67" s="7" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B68" s="7" t="s">
         <v>133</v>
-      </c>
-      <c r="B68" s="7" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2925,7 +2926,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2933,7 +2934,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2997,7 +2998,7 @@
         <v>16</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3005,7 +3006,7 @@
         <v>17</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3013,7 +3014,7 @@
         <v>18</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3021,7 +3022,7 @@
         <v>19</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3242,178 +3243,178 @@
     </row>
     <row r="51" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
More color themes for maps
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD5DF2C5-97F7-4D21-99D3-3D08D80895D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC617368-1C34-4EE6-93D3-C04F831CE6D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="337">
   <si>
     <t>exiobase</t>
   </si>
@@ -540,17 +540,522 @@
   </si>
   <si>
     <t>Stage Analysis</t>
+  </si>
+  <si>
+    <t>Region Analysis</t>
+  </si>
+  <si>
+    <t>Analyse nach Wertschöpfungsstufen</t>
+  </si>
+  <si>
+    <t>Analyse nach Regionen</t>
+  </si>
+  <si>
+    <t>World Map Settings</t>
+  </si>
+  <si>
+    <t>Erweiterte Einstellungen</t>
+  </si>
+  <si>
+    <t>Farbkarte</t>
+  </si>
+  <si>
+    <t>cm.group.perceptual</t>
+  </si>
+  <si>
+    <t>Perzeptuell</t>
+  </si>
+  <si>
+    <t>cm.group.sequential</t>
+  </si>
+  <si>
+    <t>Sequenziell</t>
+  </si>
+  <si>
+    <t>cm.group.diverging</t>
+  </si>
+  <si>
+    <t>Divergierend</t>
+  </si>
+  <si>
+    <t>cm.group.cyclic</t>
+  </si>
+  <si>
+    <t>Zyklisch</t>
+  </si>
+  <si>
+    <t>cm.group.qualitative</t>
+  </si>
+  <si>
+    <t>Qualitativ</t>
+  </si>
+  <si>
+    <t>cm.reverse</t>
+  </si>
+  <si>
+    <t>Umkehren</t>
+  </si>
+  <si>
+    <t>cmap.Reds</t>
+  </si>
+  <si>
+    <t>Rottöne</t>
+  </si>
+  <si>
+    <t>cmap.Blues</t>
+  </si>
+  <si>
+    <t>Blautöne</t>
+  </si>
+  <si>
+    <t>cmap.Greens</t>
+  </si>
+  <si>
+    <t>Grüntöne</t>
+  </si>
+  <si>
+    <t>cmap.Purples</t>
+  </si>
+  <si>
+    <t>Violettöne</t>
+  </si>
+  <si>
+    <t>cmap.Oranges</t>
+  </si>
+  <si>
+    <t>Orangetöne</t>
+  </si>
+  <si>
+    <t>cmap.Greys</t>
+  </si>
+  <si>
+    <t>Grautöne</t>
+  </si>
+  <si>
+    <t>cmap.YlGn</t>
+  </si>
+  <si>
+    <t>Gelb–Grün</t>
+  </si>
+  <si>
+    <t>cmap.YlGnBu</t>
+  </si>
+  <si>
+    <t>Gelb–Grün–Blau</t>
+  </si>
+  <si>
+    <t>cmap.GnBu</t>
+  </si>
+  <si>
+    <t>Grün–Blau</t>
+  </si>
+  <si>
+    <t>cmap.BuGn</t>
+  </si>
+  <si>
+    <t>Blau–Grün</t>
+  </si>
+  <si>
+    <t>cmap.PuBu</t>
+  </si>
+  <si>
+    <t>Violett–Blau</t>
+  </si>
+  <si>
+    <t>cmap.BuPu</t>
+  </si>
+  <si>
+    <t>Blau–Violett</t>
+  </si>
+  <si>
+    <t>cmap.OrRd</t>
+  </si>
+  <si>
+    <t>Orange–Rot</t>
+  </si>
+  <si>
+    <t>cmap.PuRd</t>
+  </si>
+  <si>
+    <t>Violett–Rot</t>
+  </si>
+  <si>
+    <t>cmap.RdPu</t>
+  </si>
+  <si>
+    <t>Rot–Violett</t>
+  </si>
+  <si>
+    <t>cmap.YlOrBr</t>
+  </si>
+  <si>
+    <t>Gelb–Orange–Braun</t>
+  </si>
+  <si>
+    <t>cmap.YlOrRd</t>
+  </si>
+  <si>
+    <t>Gelb–Orange–Rot</t>
+  </si>
+  <si>
+    <t>cmap.viridis</t>
+  </si>
+  <si>
+    <t>Viridis</t>
+  </si>
+  <si>
+    <t>cmap.plasma</t>
+  </si>
+  <si>
+    <t>Plasma</t>
+  </si>
+  <si>
+    <t>cmap.inferno</t>
+  </si>
+  <si>
+    <t>Inferno</t>
+  </si>
+  <si>
+    <t>cmap.magma</t>
+  </si>
+  <si>
+    <t>Magma</t>
+  </si>
+  <si>
+    <t>cmap.cividis</t>
+  </si>
+  <si>
+    <t>Cividis</t>
+  </si>
+  <si>
+    <t>cmap.turbo</t>
+  </si>
+  <si>
+    <t>Turbo</t>
+  </si>
+  <si>
+    <t>cmap.BrBG</t>
+  </si>
+  <si>
+    <t>Braun–Blaugrün</t>
+  </si>
+  <si>
+    <t>cmap.PiYG</t>
+  </si>
+  <si>
+    <t>Pink–Gelbgrün</t>
+  </si>
+  <si>
+    <t>cmap.PRGn</t>
+  </si>
+  <si>
+    <t>Purpur–Grün</t>
+  </si>
+  <si>
+    <t>cmap.PuOr</t>
+  </si>
+  <si>
+    <t>Violett–Orange</t>
+  </si>
+  <si>
+    <t>cmap.RdBu</t>
+  </si>
+  <si>
+    <t>Rot–Blau</t>
+  </si>
+  <si>
+    <t>cmap.RdGy</t>
+  </si>
+  <si>
+    <t>Rot–Grau</t>
+  </si>
+  <si>
+    <t>cmap.RdYlBu</t>
+  </si>
+  <si>
+    <t>Rot–Gelb–Blau</t>
+  </si>
+  <si>
+    <t>cmap.RdYlGn</t>
+  </si>
+  <si>
+    <t>Rot–Gelb–Grün</t>
+  </si>
+  <si>
+    <t>cmap.Spectral</t>
+  </si>
+  <si>
+    <t>Spektral</t>
+  </si>
+  <si>
+    <t>cmap.coolwarm</t>
+  </si>
+  <si>
+    <t>Cool–Warm</t>
+  </si>
+  <si>
+    <t>cmap.bwr</t>
+  </si>
+  <si>
+    <t>Blau–Weiß–Rot</t>
+  </si>
+  <si>
+    <t>cmap.seismic</t>
+  </si>
+  <si>
+    <t>Seismisch</t>
+  </si>
+  <si>
+    <t>cmap.twilight</t>
+  </si>
+  <si>
+    <t>Twilight</t>
+  </si>
+  <si>
+    <t>cmap.twilight_shifted</t>
+  </si>
+  <si>
+    <t>Twilight (verschoben)</t>
+  </si>
+  <si>
+    <t>cmap.hsv</t>
+  </si>
+  <si>
+    <t>HSV</t>
+  </si>
+  <si>
+    <t>cmap.tab10</t>
+  </si>
+  <si>
+    <t>Tab10</t>
+  </si>
+  <si>
+    <t>cmap.tab20</t>
+  </si>
+  <si>
+    <t>Tab20</t>
+  </si>
+  <si>
+    <t>cmap.tab20b</t>
+  </si>
+  <si>
+    <t>Tab20b</t>
+  </si>
+  <si>
+    <t>cmap.tab20c</t>
+  </si>
+  <si>
+    <t>Tab20c</t>
+  </si>
+  <si>
+    <t>cmap.Set1</t>
+  </si>
+  <si>
+    <t>Set1</t>
+  </si>
+  <si>
+    <t>cmap.Set2</t>
+  </si>
+  <si>
+    <t>Set2</t>
+  </si>
+  <si>
+    <t>cmap.Set3</t>
+  </si>
+  <si>
+    <t>Set3</t>
+  </si>
+  <si>
+    <t>cmap.Pastel1</t>
+  </si>
+  <si>
+    <t>Pastel1</t>
+  </si>
+  <si>
+    <t>cmap.Pastel2</t>
+  </si>
+  <si>
+    <t>Pastel2</t>
+  </si>
+  <si>
+    <t>cmap.Accent</t>
+  </si>
+  <si>
+    <t>Accent</t>
+  </si>
+  <si>
+    <t>cmap.Dark2</t>
+  </si>
+  <si>
+    <t>Dark2</t>
+  </si>
+  <si>
+    <t>cmap.Paired</t>
+  </si>
+  <si>
+    <t>Paired</t>
+  </si>
+  <si>
+    <t>Perceptual</t>
+  </si>
+  <si>
+    <t>Sequential</t>
+  </si>
+  <si>
+    <t>Diverging</t>
+  </si>
+  <si>
+    <t>Cyclic</t>
+  </si>
+  <si>
+    <t>Qualitative</t>
+  </si>
+  <si>
+    <t>Reverse</t>
+  </si>
+  <si>
+    <t>Reds</t>
+  </si>
+  <si>
+    <t>Blues</t>
+  </si>
+  <si>
+    <t>Greens</t>
+  </si>
+  <si>
+    <t>Purples</t>
+  </si>
+  <si>
+    <t>Oranges</t>
+  </si>
+  <si>
+    <t>Greys</t>
+  </si>
+  <si>
+    <t>YlGn</t>
+  </si>
+  <si>
+    <t>YlGnBu</t>
+  </si>
+  <si>
+    <t>GnBu</t>
+  </si>
+  <si>
+    <t>BuGn</t>
+  </si>
+  <si>
+    <t>PuBu</t>
+  </si>
+  <si>
+    <t>BuPu</t>
+  </si>
+  <si>
+    <t>OrRd</t>
+  </si>
+  <si>
+    <t>PuRd</t>
+  </si>
+  <si>
+    <t>RdPu</t>
+  </si>
+  <si>
+    <t>YlOrBr</t>
+  </si>
+  <si>
+    <t>YlOrRd</t>
+  </si>
+  <si>
+    <t>viridis</t>
+  </si>
+  <si>
+    <t>plasma</t>
+  </si>
+  <si>
+    <t>inferno</t>
+  </si>
+  <si>
+    <t>magma</t>
+  </si>
+  <si>
+    <t>cividis</t>
+  </si>
+  <si>
+    <t>turbo</t>
+  </si>
+  <si>
+    <t>BrBG</t>
+  </si>
+  <si>
+    <t>PiYG</t>
+  </si>
+  <si>
+    <t>PRGn</t>
+  </si>
+  <si>
+    <t>PuOr</t>
+  </si>
+  <si>
+    <t>RdBu</t>
+  </si>
+  <si>
+    <t>RdGy</t>
+  </si>
+  <si>
+    <t>RdYlBu</t>
+  </si>
+  <si>
+    <t>RdYlGn</t>
+  </si>
+  <si>
+    <t>Spectral</t>
+  </si>
+  <si>
+    <t>coolwarm</t>
+  </si>
+  <si>
+    <t>bwr</t>
+  </si>
+  <si>
+    <t>seismic</t>
+  </si>
+  <si>
+    <t>twilight</t>
+  </si>
+  <si>
+    <t>twilight_shifted</t>
+  </si>
+  <si>
+    <t>hsv</t>
+  </si>
+  <si>
+    <t>tab10</t>
+  </si>
+  <si>
+    <t>tab20</t>
+  </si>
+  <si>
+    <t>tab20b</t>
+  </si>
+  <si>
+    <t>tab20c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -574,6 +1079,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -626,29 +1137,32 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard 2" xfId="1" xr:uid="{C2F78208-F7F8-4542-9E5B-6270DCB86735}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
@@ -1806,15 +2320,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J88"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J148"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="115" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="60.5703125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="41.7109375" style="4" customWidth="1"/>
     <col min="3" max="6" width="9.140625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="13.5" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1822,7 +2337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="13.5" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -1830,7 +2345,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="13.5" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -1838,7 +2353,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="13.5" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -1846,7 +2361,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="13.5" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -1854,7 +2369,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="13.5" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -1862,7 +2377,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="13.5" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
@@ -1870,7 +2385,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="13.5" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
@@ -1878,7 +2393,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="13.5" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
@@ -1886,7 +2401,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="13.5" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -1894,7 +2409,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="13.5" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
@@ -1902,7 +2417,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="13.5" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -1910,7 +2425,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="13.5" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
@@ -1918,7 +2433,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="13.5" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
@@ -1926,7 +2441,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="13.5" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
@@ -1934,7 +2449,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="13.5" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
@@ -1942,7 +2457,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.5" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>17</v>
       </c>
@@ -1950,7 +2465,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="13.5" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
@@ -1958,7 +2473,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="13.5" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>19</v>
       </c>
@@ -1966,7 +2481,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="13.5" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -1974,7 +2489,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ht="13.5" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>21</v>
       </c>
@@ -1982,7 +2497,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ht="13.5" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>22</v>
       </c>
@@ -1990,7 +2505,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ht="13.5" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>23</v>
       </c>
@@ -1998,7 +2513,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="13.5" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>24</v>
       </c>
@@ -2006,7 +2521,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" ht="13.5" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>25</v>
       </c>
@@ -2014,7 +2529,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" ht="13.5" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>26</v>
       </c>
@@ -2022,7 +2537,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" ht="13.5" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>27</v>
       </c>
@@ -2030,7 +2545,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" ht="13.5" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>28</v>
       </c>
@@ -2038,7 +2553,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" ht="13.5" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>29</v>
       </c>
@@ -2046,7 +2561,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" ht="13.5" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>30</v>
       </c>
@@ -2054,7 +2569,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" ht="13.5" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>31</v>
       </c>
@@ -2062,7 +2577,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" ht="13.5" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>32</v>
       </c>
@@ -2070,7 +2585,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" ht="13.5" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>33</v>
       </c>
@@ -2078,7 +2593,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" ht="13.5" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>34</v>
       </c>
@@ -2086,7 +2601,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" ht="13.5" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>35</v>
       </c>
@@ -2094,7 +2609,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" ht="13.5" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>36</v>
       </c>
@@ -2102,7 +2617,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" ht="13.5" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>37</v>
       </c>
@@ -2110,7 +2625,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" ht="13.5" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>38</v>
       </c>
@@ -2118,7 +2633,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" ht="13.5" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>39</v>
       </c>
@@ -2126,7 +2641,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" ht="13.5" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>40</v>
       </c>
@@ -2134,7 +2649,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" ht="13.5" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>41</v>
       </c>
@@ -2142,7 +2657,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" ht="13.5" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>42</v>
       </c>
@@ -2150,7 +2665,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" ht="13.5" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>43</v>
       </c>
@@ -2158,7 +2673,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" ht="15.95" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>44</v>
       </c>
@@ -2166,7 +2681,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" ht="15.95" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>46</v>
       </c>
@@ -2174,7 +2689,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" ht="15.95" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>19</v>
       </c>
@@ -2182,7 +2697,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" ht="15" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>92</v>
       </c>
@@ -2190,7 +2705,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" ht="15" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>94</v>
       </c>
@@ -2198,7 +2713,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" ht="15" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>96</v>
       </c>
@@ -2206,7 +2721,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" ht="15" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>98</v>
       </c>
@@ -2214,7 +2729,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" ht="15" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>100</v>
       </c>
@@ -2222,7 +2737,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" ht="15" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>102</v>
       </c>
@@ -2230,7 +2745,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" ht="15" customHeight="1">
       <c r="A53" s="4" t="s">
         <v>104</v>
       </c>
@@ -2238,7 +2753,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" ht="15" customHeight="1">
       <c r="A54" s="4" t="s">
         <v>106</v>
       </c>
@@ -2246,7 +2761,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" ht="15" customHeight="1">
       <c r="A55" s="4" t="s">
         <v>108</v>
       </c>
@@ -2254,7 +2769,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" ht="15" customHeight="1">
       <c r="A56" s="4" t="s">
         <v>110</v>
       </c>
@@ -2262,7 +2777,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" ht="15" customHeight="1">
       <c r="A57" s="4" t="s">
         <v>112</v>
       </c>
@@ -2270,7 +2785,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" ht="15" customHeight="1">
       <c r="A58" s="4" t="s">
         <v>113</v>
       </c>
@@ -2278,7 +2793,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" ht="15" customHeight="1">
       <c r="A59" s="4" t="s">
         <v>118</v>
       </c>
@@ -2286,7 +2801,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" ht="15" customHeight="1">
       <c r="A60" s="4" t="s">
         <v>116</v>
       </c>
@@ -2294,7 +2809,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" ht="15" customHeight="1">
       <c r="A61" s="4" t="s">
         <v>117</v>
       </c>
@@ -2302,7 +2817,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" ht="15" customHeight="1">
       <c r="A62" s="4" t="s">
         <v>120</v>
       </c>
@@ -2318,7 +2833,7 @@
       <c r="I62" s="8"/>
       <c r="J62" s="8"/>
     </row>
-    <row r="63" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" ht="15" customHeight="1">
       <c r="A63" s="7" t="s">
         <v>122</v>
       </c>
@@ -2326,7 +2841,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" ht="15" customHeight="1">
       <c r="A64" s="7" t="s">
         <v>124</v>
       </c>
@@ -2334,7 +2849,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" ht="15" customHeight="1">
       <c r="A65" s="9" t="s">
         <v>126</v>
       </c>
@@ -2342,7 +2857,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" ht="15" customHeight="1">
       <c r="A66" s="4" t="s">
         <v>129</v>
       </c>
@@ -2350,7 +2865,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" ht="15" customHeight="1">
       <c r="A67" s="4" t="s">
         <v>130</v>
       </c>
@@ -2358,7 +2873,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" ht="15" customHeight="1">
       <c r="A68" s="7" t="s">
         <v>132</v>
       </c>
@@ -2366,7 +2881,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" ht="15" customHeight="1">
       <c r="A69" s="4" t="s">
         <v>135</v>
       </c>
@@ -2374,7 +2889,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" ht="15" customHeight="1">
       <c r="A70" s="4" t="s">
         <v>137</v>
       </c>
@@ -2382,7 +2897,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" ht="15" customHeight="1">
       <c r="A71" s="4" t="s">
         <v>138</v>
       </c>
@@ -2390,7 +2905,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" ht="15" customHeight="1">
       <c r="A72" s="4" t="s">
         <v>139</v>
       </c>
@@ -2398,7 +2913,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" ht="15" customHeight="1">
       <c r="A73" s="4" t="s">
         <v>140</v>
       </c>
@@ -2406,7 +2921,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" ht="15" customHeight="1">
       <c r="A74" s="4" t="s">
         <v>141</v>
       </c>
@@ -2414,7 +2929,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" ht="15" customHeight="1">
       <c r="A75" s="4" t="s">
         <v>142</v>
       </c>
@@ -2422,7 +2937,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" ht="15" customHeight="1">
       <c r="A76" s="4" t="s">
         <v>143</v>
       </c>
@@ -2430,7 +2945,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" ht="15" customHeight="1">
       <c r="A77" s="4" t="s">
         <v>144</v>
       </c>
@@ -2438,7 +2953,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" ht="15" customHeight="1">
       <c r="A78" s="4" t="s">
         <v>145</v>
       </c>
@@ -2446,7 +2961,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" ht="15" customHeight="1">
       <c r="A79" s="4" t="s">
         <v>146</v>
       </c>
@@ -2454,7 +2969,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" ht="15" customHeight="1">
       <c r="A80" s="4" t="s">
         <v>147</v>
       </c>
@@ -2462,7 +2977,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" ht="15" customHeight="1">
       <c r="A81" s="4" t="s">
         <v>148</v>
       </c>
@@ -2470,7 +2985,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" ht="15" customHeight="1">
       <c r="A82" s="4" t="s">
         <v>149</v>
       </c>
@@ -2478,7 +2993,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" ht="15" customHeight="1">
       <c r="A83" s="4" t="s">
         <v>150</v>
       </c>
@@ -2486,7 +3001,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" ht="15" customHeight="1">
       <c r="A84" s="4" t="s">
         <v>151</v>
       </c>
@@ -2494,7 +3009,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" ht="15" customHeight="1">
       <c r="A85" s="4" t="s">
         <v>162</v>
       </c>
@@ -2502,7 +3017,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" ht="15" customHeight="1">
       <c r="A86" s="4" t="s">
         <v>163</v>
       </c>
@@ -2510,7 +3025,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" ht="15" customHeight="1">
       <c r="A87" s="4" t="s">
         <v>164</v>
       </c>
@@ -2518,12 +3033,492 @@
         <v>164</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" ht="15" customHeight="1">
       <c r="A88" s="4" t="s">
         <v>165</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>165</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" ht="15" customHeight="1">
+      <c r="A89" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" ht="15" customHeight="1">
+      <c r="A90" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" ht="15" customHeight="1">
+      <c r="A91" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" ht="15" customHeight="1">
+      <c r="A92" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" ht="15" customHeight="1">
+      <c r="A93" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" ht="15" customHeight="1">
+      <c r="A94" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" ht="15" customHeight="1">
+      <c r="A95" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" ht="15" customHeight="1">
+      <c r="A96" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" ht="15" customHeight="1">
+      <c r="A97" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="15" customHeight="1">
+      <c r="A98" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" ht="15" customHeight="1">
+      <c r="A99" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" ht="15" customHeight="1">
+      <c r="A100" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" ht="15" customHeight="1">
+      <c r="A101" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" ht="15" customHeight="1">
+      <c r="A102" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" ht="15" customHeight="1">
+      <c r="A103" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" ht="15" customHeight="1">
+      <c r="A104" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" ht="15" customHeight="1">
+      <c r="A105" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" ht="15" customHeight="1">
+      <c r="A106" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" ht="15" customHeight="1">
+      <c r="A107" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" ht="15" customHeight="1">
+      <c r="A108" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" ht="15" customHeight="1">
+      <c r="A109" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" ht="15" customHeight="1">
+      <c r="A110" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" ht="15" customHeight="1">
+      <c r="A111" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" ht="15" customHeight="1">
+      <c r="A112" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" ht="15" customHeight="1">
+      <c r="A113" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" ht="15" customHeight="1">
+      <c r="A114" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" ht="15" customHeight="1">
+      <c r="A115" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" ht="15" customHeight="1">
+      <c r="A116" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" ht="15" customHeight="1">
+      <c r="A117" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" ht="15" customHeight="1">
+      <c r="A118" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" ht="15" customHeight="1">
+      <c r="A119" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" ht="15" customHeight="1">
+      <c r="A120" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" ht="15" customHeight="1">
+      <c r="A121" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" ht="15" customHeight="1">
+      <c r="A122" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" ht="15" customHeight="1">
+      <c r="A123" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" ht="15" customHeight="1">
+      <c r="A124" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" ht="15" customHeight="1">
+      <c r="A125" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" ht="15" customHeight="1">
+      <c r="A126" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" ht="15" customHeight="1">
+      <c r="A127" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" ht="15" customHeight="1">
+      <c r="A128" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" ht="15" customHeight="1">
+      <c r="A129" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" ht="15" customHeight="1">
+      <c r="A130" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" ht="15" customHeight="1">
+      <c r="A131" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" ht="15" customHeight="1">
+      <c r="A132" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" ht="15" customHeight="1">
+      <c r="A133" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" ht="15" customHeight="1">
+      <c r="A134" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" ht="15" customHeight="1">
+      <c r="A135" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" ht="15" customHeight="1">
+      <c r="A136" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" ht="15" customHeight="1">
+      <c r="A137" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" ht="15" customHeight="1">
+      <c r="A138" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" ht="15" customHeight="1">
+      <c r="A139" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" ht="15" customHeight="1">
+      <c r="A140" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" ht="15" customHeight="1">
+      <c r="A141" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" ht="15" customHeight="1">
+      <c r="A142" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" ht="15" customHeight="1">
+      <c r="A143" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" ht="15" customHeight="1">
+      <c r="A144" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" ht="15" customHeight="1">
+      <c r="A145" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" ht="15" customHeight="1">
+      <c r="A146" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" ht="15" customHeight="1">
+      <c r="A147" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" ht="15" customHeight="1">
+      <c r="A148" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -2537,16 +3532,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B89"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B148"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="115" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="75" style="4" customWidth="1"/>
+    <col min="1" max="1" width="54.140625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="54.28515625" style="4" customWidth="1"/>
     <col min="3" max="6" width="9.140625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="13.5" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2554,7 +3549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="13.5" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -2562,7 +3557,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="13.5" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -2570,7 +3565,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="13.5" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -2578,7 +3573,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="13.5" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -2586,7 +3581,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="30">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -2594,7 +3589,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
@@ -2602,7 +3597,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="45" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
@@ -2610,7 +3605,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="30" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
@@ -2618,7 +3613,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="13.5" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>11</v>
       </c>
@@ -2626,7 +3621,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="13.5" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -2634,7 +3629,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="13.5" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -2642,7 +3637,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="13.5" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
@@ -2650,7 +3645,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="13.5" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
@@ -2658,7 +3653,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="13.5" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
@@ -2666,7 +3661,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="13.5" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
@@ -2674,7 +3669,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.5" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>17</v>
       </c>
@@ -2682,7 +3677,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="13.5" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
@@ -2690,7 +3685,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="13.5" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>19</v>
       </c>
@@ -2698,7 +3693,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="13.5" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -2706,7 +3701,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ht="13.5" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>21</v>
       </c>
@@ -2714,7 +3709,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ht="13.5" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>22</v>
       </c>
@@ -2722,7 +3717,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ht="13.5" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>23</v>
       </c>
@@ -2730,7 +3725,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="13.5" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>24</v>
       </c>
@@ -2738,7 +3733,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" ht="13.5" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>25</v>
       </c>
@@ -2746,7 +3741,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" ht="13.5" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>26</v>
       </c>
@@ -2754,7 +3749,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" ht="13.5" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>27</v>
       </c>
@@ -2762,7 +3757,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" ht="13.5" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>28</v>
       </c>
@@ -2770,7 +3765,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" ht="13.5" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>29</v>
       </c>
@@ -2778,7 +3773,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" ht="13.5" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>30</v>
       </c>
@@ -2786,7 +3781,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" ht="13.5" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>31</v>
       </c>
@@ -2794,7 +3789,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" ht="13.5" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>32</v>
       </c>
@@ -2802,7 +3797,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" ht="13.5" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>33</v>
       </c>
@@ -2810,7 +3805,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" ht="13.5" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>34</v>
       </c>
@@ -2818,7 +3813,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" ht="13.5" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>35</v>
       </c>
@@ -2826,7 +3821,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" ht="13.5" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>36</v>
       </c>
@@ -2834,7 +3829,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" ht="13.5" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>37</v>
       </c>
@@ -2842,7 +3837,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" ht="13.5" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>38</v>
       </c>
@@ -2850,7 +3845,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" ht="13.5" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>39</v>
       </c>
@@ -2858,7 +3853,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" ht="13.5" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>40</v>
       </c>
@@ -2866,7 +3861,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" ht="13.5" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>41</v>
       </c>
@@ -2874,7 +3869,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" ht="13.5" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>42</v>
       </c>
@@ -2882,7 +3877,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" ht="13.5" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>43</v>
       </c>
@@ -2890,7 +3885,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" ht="15.95" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>44</v>
       </c>
@@ -2898,7 +3893,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" ht="15.95" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>46</v>
       </c>
@@ -2906,7 +3901,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" ht="15.95" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>19</v>
       </c>
@@ -2914,7 +3909,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" ht="15" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>92</v>
       </c>
@@ -2922,7 +3917,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" ht="15" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>94</v>
       </c>
@@ -2930,7 +3925,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" ht="15" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>96</v>
       </c>
@@ -2938,7 +3933,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" ht="15" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>98</v>
       </c>
@@ -2946,7 +3941,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" ht="15" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>100</v>
       </c>
@@ -2954,7 +3949,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" ht="15" customHeight="1">
       <c r="A52" s="4" t="s">
         <v>102</v>
       </c>
@@ -2962,7 +3957,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" ht="15" customHeight="1">
       <c r="A53" s="4" t="s">
         <v>104</v>
       </c>
@@ -2970,7 +3965,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" ht="15" customHeight="1">
       <c r="A54" s="4" t="s">
         <v>106</v>
       </c>
@@ -2978,7 +3973,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" ht="15" customHeight="1">
       <c r="A55" s="4" t="s">
         <v>108</v>
       </c>
@@ -2986,7 +3981,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" ht="15" customHeight="1">
       <c r="A56" s="4" t="s">
         <v>110</v>
       </c>
@@ -2994,7 +3989,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" ht="15" customHeight="1">
       <c r="A57" s="4" t="s">
         <v>112</v>
       </c>
@@ -3002,7 +3997,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" ht="15" customHeight="1">
       <c r="A58" s="4" t="s">
         <v>113</v>
       </c>
@@ -3010,7 +4005,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" ht="15" customHeight="1">
       <c r="A59" s="4" t="s">
         <v>118</v>
       </c>
@@ -3018,7 +4013,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" ht="15" customHeight="1">
       <c r="A60" s="4" t="s">
         <v>116</v>
       </c>
@@ -3026,7 +4021,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" ht="15" customHeight="1">
       <c r="A61" s="4" t="s">
         <v>117</v>
       </c>
@@ -3034,7 +4029,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" ht="15" customHeight="1">
       <c r="A62" s="4" t="s">
         <v>120</v>
       </c>
@@ -3042,7 +4037,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" ht="15" customHeight="1">
       <c r="A63" s="7" t="s">
         <v>122</v>
       </c>
@@ -3050,7 +4045,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" ht="15" customHeight="1">
       <c r="A64" s="7" t="s">
         <v>124</v>
       </c>
@@ -3058,7 +4053,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" ht="15" customHeight="1">
       <c r="A65" s="4" t="s">
         <v>126</v>
       </c>
@@ -3066,7 +4061,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" ht="15" customHeight="1">
       <c r="A66" s="4" t="s">
         <v>129</v>
       </c>
@@ -3074,7 +4069,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" ht="15" customHeight="1">
       <c r="A67" s="4" t="s">
         <v>130</v>
       </c>
@@ -3082,7 +4077,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" ht="15" customHeight="1">
       <c r="A68" s="7" t="s">
         <v>132</v>
       </c>
@@ -3090,7 +4085,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" ht="15" customHeight="1">
       <c r="A69" s="4" t="s">
         <v>135</v>
       </c>
@@ -3098,7 +4093,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" ht="15" customHeight="1">
       <c r="A70" s="4" t="s">
         <v>137</v>
       </c>
@@ -3106,7 +4101,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" ht="15" customHeight="1">
       <c r="A71" s="4" t="s">
         <v>138</v>
       </c>
@@ -3114,7 +4109,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" ht="15" customHeight="1">
       <c r="A72" s="4" t="s">
         <v>139</v>
       </c>
@@ -3122,7 +4117,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" ht="15" customHeight="1">
       <c r="A73" s="4" t="s">
         <v>140</v>
       </c>
@@ -3130,7 +4125,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" ht="15" customHeight="1">
       <c r="A74" s="4" t="s">
         <v>141</v>
       </c>
@@ -3138,7 +4133,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" ht="15" customHeight="1">
       <c r="A75" s="4" t="s">
         <v>142</v>
       </c>
@@ -3146,7 +4141,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" ht="15" customHeight="1">
       <c r="A76" s="4" t="s">
         <v>143</v>
       </c>
@@ -3154,7 +4149,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" ht="15" customHeight="1">
       <c r="A77" s="4" t="s">
         <v>144</v>
       </c>
@@ -3162,7 +4157,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" ht="15" customHeight="1">
       <c r="A78" s="4" t="s">
         <v>145</v>
       </c>
@@ -3170,7 +4165,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" ht="15" customHeight="1">
       <c r="A79" s="4" t="s">
         <v>146</v>
       </c>
@@ -3178,7 +4173,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" ht="15" customHeight="1">
       <c r="A80" s="4" t="s">
         <v>147</v>
       </c>
@@ -3186,7 +4181,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" ht="15" customHeight="1">
       <c r="A81" s="4" t="s">
         <v>148</v>
       </c>
@@ -3194,7 +4189,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" ht="15" customHeight="1">
       <c r="A82" s="4" t="s">
         <v>149</v>
       </c>
@@ -3202,7 +4197,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" ht="15" customHeight="1">
       <c r="A83" s="4" t="s">
         <v>150</v>
       </c>
@@ -3210,7 +4205,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" ht="15" customHeight="1">
       <c r="A84" s="4" t="s">
         <v>151</v>
       </c>
@@ -3218,7 +4213,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" ht="15" customHeight="1">
       <c r="A85" s="4" t="s">
         <v>162</v>
       </c>
@@ -3226,7 +4221,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" ht="15" customHeight="1">
       <c r="A86" s="4" t="s">
         <v>163</v>
       </c>
@@ -3234,7 +4229,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" ht="15" customHeight="1">
       <c r="A87" s="4" t="s">
         <v>164</v>
       </c>
@@ -3242,7 +4237,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" ht="15" customHeight="1">
       <c r="A88" s="4" t="s">
         <v>165</v>
       </c>
@@ -3250,14 +4245,489 @@
         <v>169</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" ht="15" customHeight="1">
       <c r="A89" s="4" t="s">
         <v>170</v>
       </c>
+      <c r="B89" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" ht="15" customHeight="1">
+      <c r="A90" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" ht="15" customHeight="1">
+      <c r="A91" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" ht="15" customHeight="1">
+      <c r="A92" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" ht="15" customHeight="1">
+      <c r="A93" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" ht="15" customHeight="1">
+      <c r="A94" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" ht="15" customHeight="1">
+      <c r="A95" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" ht="15" customHeight="1">
+      <c r="A96" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" ht="15" customHeight="1">
+      <c r="A97" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="15" customHeight="1">
+      <c r="A98" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" ht="15" customHeight="1">
+      <c r="A99" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" ht="15" customHeight="1">
+      <c r="A100" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" ht="15" customHeight="1">
+      <c r="A101" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" ht="15" customHeight="1">
+      <c r="A102" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" ht="15" customHeight="1">
+      <c r="A103" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" ht="15" customHeight="1">
+      <c r="A104" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" ht="15" customHeight="1">
+      <c r="A105" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" ht="15" customHeight="1">
+      <c r="A106" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" ht="15" customHeight="1">
+      <c r="A107" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" ht="15" customHeight="1">
+      <c r="A108" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" ht="15" customHeight="1">
+      <c r="A109" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" ht="15" customHeight="1">
+      <c r="A110" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" ht="15" customHeight="1">
+      <c r="A111" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" ht="15" customHeight="1">
+      <c r="A112" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" ht="15" customHeight="1">
+      <c r="A113" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" ht="15" customHeight="1">
+      <c r="A114" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" ht="15" customHeight="1">
+      <c r="A115" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" ht="15" customHeight="1">
+      <c r="A116" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" ht="15" customHeight="1">
+      <c r="A117" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" ht="15" customHeight="1">
+      <c r="A118" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" ht="15" customHeight="1">
+      <c r="A119" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" ht="15" customHeight="1">
+      <c r="A120" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" ht="15" customHeight="1">
+      <c r="A121" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" ht="15" customHeight="1">
+      <c r="A122" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" ht="15" customHeight="1">
+      <c r="A123" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" ht="15" customHeight="1">
+      <c r="A124" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" ht="15" customHeight="1">
+      <c r="A125" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" ht="15" customHeight="1">
+      <c r="A126" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" ht="15" customHeight="1">
+      <c r="A127" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" ht="15" customHeight="1">
+      <c r="A128" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" ht="15" customHeight="1">
+      <c r="A129" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" ht="15" customHeight="1">
+      <c r="A130" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" ht="15" customHeight="1">
+      <c r="A131" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" ht="15" customHeight="1">
+      <c r="A132" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" ht="15" customHeight="1">
+      <c r="A133" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" ht="15" customHeight="1">
+      <c r="A134" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" ht="15" customHeight="1">
+      <c r="A135" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" ht="15" customHeight="1">
+      <c r="A136" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" ht="15" customHeight="1">
+      <c r="A137" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" ht="15" customHeight="1">
+      <c r="A138" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" ht="15" customHeight="1">
+      <c r="A139" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" ht="15" customHeight="1">
+      <c r="A140" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" ht="15" customHeight="1">
+      <c r="A141" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" ht="15" customHeight="1">
+      <c r="A142" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" ht="15" customHeight="1">
+      <c r="A143" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" ht="15" customHeight="1">
+      <c r="A144" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" ht="15" customHeight="1">
+      <c r="A145" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" ht="15" customHeight="1">
+      <c r="A146" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" ht="15" customHeight="1">
+      <c r="A147" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" ht="15" customHeight="1">
+      <c r="A148" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>288</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -3266,15 +4736,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B92"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B152"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="115" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="64" style="4" customWidth="1"/>
+    <col min="2" max="2" width="49.85546875" style="4" customWidth="1"/>
     <col min="3" max="6" width="9.140625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="13.5" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -3282,7 +4753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="13.5" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -3290,7 +4761,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="13.5" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -3298,7 +4769,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="13.5" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -3306,7 +4777,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="13.5" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -3314,7 +4785,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="13.5" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -3322,7 +4793,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="13.5" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
@@ -3330,7 +4801,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="13.5" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
@@ -3338,7 +4809,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="13.5" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
@@ -3346,7 +4817,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="13.5" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -3354,7 +4825,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="13.5" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
@@ -3362,7 +4833,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="13.5" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3370,7 +4841,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="13.5" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
@@ -3378,7 +4849,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="13.5" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
@@ -3386,7 +4857,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="13.5" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
@@ -3394,7 +4865,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="13.5" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
@@ -3402,7 +4873,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.5" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>17</v>
       </c>
@@ -3410,7 +4881,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="13.5" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
@@ -3418,7 +4889,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="13.5" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>19</v>
       </c>
@@ -3426,7 +4897,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="13.5" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
@@ -3434,7 +4905,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ht="13.5" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
@@ -3442,7 +4913,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ht="13.5" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
@@ -3450,7 +4921,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ht="13.5" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>19</v>
       </c>
@@ -3458,7 +4929,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="13.5" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -3466,7 +4937,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" ht="13.5" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>21</v>
       </c>
@@ -3474,7 +4945,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" ht="13.5" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>22</v>
       </c>
@@ -3482,7 +4953,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" ht="13.5" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>23</v>
       </c>
@@ -3490,7 +4961,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" ht="13.5" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>24</v>
       </c>
@@ -3498,7 +4969,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" ht="13.5" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>25</v>
       </c>
@@ -3506,7 +4977,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" ht="13.5" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>26</v>
       </c>
@@ -3514,7 +4985,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" ht="13.5" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>27</v>
       </c>
@@ -3522,7 +4993,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" ht="13.5" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>28</v>
       </c>
@@ -3530,7 +5001,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" ht="13.5" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>29</v>
       </c>
@@ -3538,7 +5009,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" ht="13.5" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>30</v>
       </c>
@@ -3546,7 +5017,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" ht="13.5" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>31</v>
       </c>
@@ -3554,7 +5025,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" ht="13.5" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>32</v>
       </c>
@@ -3562,7 +5033,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" ht="13.5" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>33</v>
       </c>
@@ -3570,7 +5041,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" ht="13.5" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>34</v>
       </c>
@@ -3578,7 +5049,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" ht="13.5" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>35</v>
       </c>
@@ -3586,7 +5057,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" ht="13.5" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>36</v>
       </c>
@@ -3594,7 +5065,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" ht="13.5" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>37</v>
       </c>
@@ -3602,7 +5073,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" ht="13.5" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>38</v>
       </c>
@@ -3610,7 +5081,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" ht="13.5" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>39</v>
       </c>
@@ -3618,7 +5089,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" ht="13.5" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>40</v>
       </c>
@@ -3626,7 +5097,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" ht="13.5" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>41</v>
       </c>
@@ -3634,7 +5105,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" ht="13.5" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>42</v>
       </c>
@@ -3642,7 +5113,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" ht="13.5" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>43</v>
       </c>
@@ -3650,7 +5121,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" ht="15.95" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>44</v>
       </c>
@@ -3658,7 +5129,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" ht="15.95" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>46</v>
       </c>
@@ -3666,7 +5137,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" ht="15.95" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>19</v>
       </c>
@@ -3674,7 +5145,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" ht="15" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>92</v>
       </c>
@@ -3682,7 +5153,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" ht="15" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>94</v>
       </c>
@@ -3690,7 +5161,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" ht="15" customHeight="1">
       <c r="A53" s="2" t="s">
         <v>96</v>
       </c>
@@ -3698,7 +5169,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" ht="15" customHeight="1">
       <c r="A54" s="2" t="s">
         <v>98</v>
       </c>
@@ -3706,7 +5177,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" ht="15" customHeight="1">
       <c r="A55" s="2" t="s">
         <v>100</v>
       </c>
@@ -3714,7 +5185,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" ht="15" customHeight="1">
       <c r="A56" s="4" t="s">
         <v>102</v>
       </c>
@@ -3722,7 +5193,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" ht="15" customHeight="1">
       <c r="A57" s="4" t="s">
         <v>104</v>
       </c>
@@ -3730,7 +5201,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" ht="15" customHeight="1">
       <c r="A58" s="4" t="s">
         <v>106</v>
       </c>
@@ -3738,7 +5209,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" ht="15" customHeight="1">
       <c r="A59" s="4" t="s">
         <v>108</v>
       </c>
@@ -3746,7 +5217,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" ht="15" customHeight="1">
       <c r="A60" s="4" t="s">
         <v>110</v>
       </c>
@@ -3754,7 +5225,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" ht="15" customHeight="1">
       <c r="A61" s="4" t="s">
         <v>112</v>
       </c>
@@ -3762,7 +5233,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" ht="15" customHeight="1">
       <c r="A62" s="4" t="s">
         <v>113</v>
       </c>
@@ -3770,7 +5241,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" ht="15" customHeight="1">
       <c r="A63" s="4" t="s">
         <v>118</v>
       </c>
@@ -3778,7 +5249,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" ht="15" customHeight="1">
       <c r="A64" s="4" t="s">
         <v>116</v>
       </c>
@@ -3786,7 +5257,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" ht="15" customHeight="1">
       <c r="A65" s="4" t="s">
         <v>117</v>
       </c>
@@ -3794,7 +5265,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" ht="15" customHeight="1">
       <c r="A66" s="4" t="s">
         <v>120</v>
       </c>
@@ -3802,7 +5273,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" ht="15" customHeight="1">
       <c r="A67" s="7" t="s">
         <v>122</v>
       </c>
@@ -3810,7 +5281,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" ht="15" customHeight="1">
       <c r="A68" s="7" t="s">
         <v>124</v>
       </c>
@@ -3818,7 +5289,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" ht="15" customHeight="1">
       <c r="A69" s="4" t="s">
         <v>126</v>
       </c>
@@ -3826,7 +5297,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" ht="15" customHeight="1">
       <c r="A70" s="4" t="s">
         <v>129</v>
       </c>
@@ -3834,7 +5305,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" ht="15" customHeight="1">
       <c r="A71" s="4" t="s">
         <v>130</v>
       </c>
@@ -3842,7 +5313,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" ht="15" customHeight="1">
       <c r="A72" s="7" t="s">
         <v>132</v>
       </c>
@@ -3850,7 +5321,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" ht="15" customHeight="1">
       <c r="A73" s="4" t="s">
         <v>135</v>
       </c>
@@ -3858,7 +5329,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" ht="15" customHeight="1">
       <c r="A74" s="4" t="s">
         <v>137</v>
       </c>
@@ -3866,7 +5337,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" ht="15" customHeight="1">
       <c r="A75" s="4" t="s">
         <v>138</v>
       </c>
@@ -3874,7 +5345,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" ht="15" customHeight="1">
       <c r="A76" s="4" t="s">
         <v>139</v>
       </c>
@@ -3882,7 +5353,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" ht="15" customHeight="1">
       <c r="A77" s="4" t="s">
         <v>140</v>
       </c>
@@ -3890,7 +5361,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" ht="15" customHeight="1">
       <c r="A78" s="4" t="s">
         <v>141</v>
       </c>
@@ -3898,7 +5369,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" ht="15" customHeight="1">
       <c r="A79" s="4" t="s">
         <v>142</v>
       </c>
@@ -3906,7 +5377,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" ht="15" customHeight="1">
       <c r="A80" s="4" t="s">
         <v>143</v>
       </c>
@@ -3914,7 +5385,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" ht="15" customHeight="1">
       <c r="A81" s="4" t="s">
         <v>144</v>
       </c>
@@ -3922,7 +5393,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" ht="15" customHeight="1">
       <c r="A82" s="4" t="s">
         <v>145</v>
       </c>
@@ -3930,7 +5401,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" ht="15" customHeight="1">
       <c r="A83" s="4" t="s">
         <v>146</v>
       </c>
@@ -3938,7 +5409,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" ht="15" customHeight="1">
       <c r="A84" s="4" t="s">
         <v>147</v>
       </c>
@@ -3946,7 +5417,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" ht="15" customHeight="1">
       <c r="A85" s="4" t="s">
         <v>148</v>
       </c>
@@ -3954,7 +5425,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" ht="15" customHeight="1">
       <c r="A86" s="4" t="s">
         <v>149</v>
       </c>
@@ -3962,7 +5433,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" ht="15" customHeight="1">
       <c r="A87" s="4" t="s">
         <v>150</v>
       </c>
@@ -3970,7 +5441,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" ht="15" customHeight="1">
       <c r="A88" s="4" t="s">
         <v>151</v>
       </c>
@@ -3978,7 +5449,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" ht="15" customHeight="1">
       <c r="A89" s="4" t="s">
         <v>162</v>
       </c>
@@ -3986,7 +5457,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="90" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" ht="15" customHeight="1">
       <c r="A90" s="4" t="s">
         <v>163</v>
       </c>
@@ -3994,7 +5465,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" ht="15" customHeight="1">
       <c r="A91" s="4" t="s">
         <v>164</v>
       </c>
@@ -4002,12 +5473,492 @@
         <v>164</v>
       </c>
     </row>
-    <row r="92" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" ht="15" customHeight="1">
       <c r="A92" s="4" t="s">
         <v>165</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>165</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" ht="15" customHeight="1">
+      <c r="A93" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" ht="15" customHeight="1">
+      <c r="A94" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" ht="15" customHeight="1">
+      <c r="A95" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" ht="15" customHeight="1">
+      <c r="A96" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" ht="15" customHeight="1">
+      <c r="A97" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="15" customHeight="1">
+      <c r="A98" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" ht="15" customHeight="1">
+      <c r="A99" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" ht="15" customHeight="1">
+      <c r="A100" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" ht="15" customHeight="1">
+      <c r="A101" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" ht="15" customHeight="1">
+      <c r="A102" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" ht="15" customHeight="1">
+      <c r="A103" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" ht="15" customHeight="1">
+      <c r="A104" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" ht="15" customHeight="1">
+      <c r="A105" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" ht="15" customHeight="1">
+      <c r="A106" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" ht="15" customHeight="1">
+      <c r="A107" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" ht="15" customHeight="1">
+      <c r="A108" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" ht="15" customHeight="1">
+      <c r="A109" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" ht="15" customHeight="1">
+      <c r="A110" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" ht="15" customHeight="1">
+      <c r="A111" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" ht="15" customHeight="1">
+      <c r="A112" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" ht="15" customHeight="1">
+      <c r="A113" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" ht="15" customHeight="1">
+      <c r="A114" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" ht="15" customHeight="1">
+      <c r="A115" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" ht="15" customHeight="1">
+      <c r="A116" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" ht="15" customHeight="1">
+      <c r="A117" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" ht="15" customHeight="1">
+      <c r="A118" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" ht="15" customHeight="1">
+      <c r="A119" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" ht="15" customHeight="1">
+      <c r="A120" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" ht="15" customHeight="1">
+      <c r="A121" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" ht="15" customHeight="1">
+      <c r="A122" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" ht="15" customHeight="1">
+      <c r="A123" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" ht="15" customHeight="1">
+      <c r="A124" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" ht="15" customHeight="1">
+      <c r="A125" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" ht="15" customHeight="1">
+      <c r="A126" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" ht="15" customHeight="1">
+      <c r="A127" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" ht="15" customHeight="1">
+      <c r="A128" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" ht="15" customHeight="1">
+      <c r="A129" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" ht="15" customHeight="1">
+      <c r="A130" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" ht="15" customHeight="1">
+      <c r="A131" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" ht="15" customHeight="1">
+      <c r="A132" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" ht="15" customHeight="1">
+      <c r="A133" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" ht="15" customHeight="1">
+      <c r="A134" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" ht="15" customHeight="1">
+      <c r="A135" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" ht="15" customHeight="1">
+      <c r="A136" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" ht="15" customHeight="1">
+      <c r="A137" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" ht="15" customHeight="1">
+      <c r="A138" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" ht="15" customHeight="1">
+      <c r="A139" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" ht="15" customHeight="1">
+      <c r="A140" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" ht="15" customHeight="1">
+      <c r="A141" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" ht="15" customHeight="1">
+      <c r="A142" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" ht="15" customHeight="1">
+      <c r="A143" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" ht="15" customHeight="1">
+      <c r="A144" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" ht="15" customHeight="1">
+      <c r="A145" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" ht="15" customHeight="1">
+      <c r="A146" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" ht="15" customHeight="1">
+      <c r="A147" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" ht="15" customHeight="1">
+      <c r="A148" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" ht="15" customHeight="1">
+      <c r="A149" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" ht="15" customHeight="1">
+      <c r="A150" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" ht="15" customHeight="1">
+      <c r="A151" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" ht="15" customHeight="1">
+      <c r="A152" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B152" s="4" t="s">
+        <v>288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added detailed docstring and comments
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F860D9-EE59-4432-BAE2-28EDC65D346E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59270F15-0AB1-49CD-A204-08B043228A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1012" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="403">
   <si>
     <t>exiobase</t>
   </si>
@@ -1161,6 +1161,81 @@
   </si>
   <si>
     <t>Wähle bis zu 3 Impacts zum Vergleichen aus.</t>
+  </si>
+  <si>
+    <t>Einstellungen öffnen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Akzent </t>
+  </si>
+  <si>
+    <t>Dunkel 2</t>
+  </si>
+  <si>
+    <t>Open settings</t>
+  </si>
+  <si>
+    <t>Refresh</t>
+  </si>
+  <si>
+    <t>Export data</t>
+  </si>
+  <si>
+    <t>Aktualisieren</t>
+  </si>
+  <si>
+    <t>Daten exportieren</t>
+  </si>
+  <si>
+    <t>Impacts</t>
+  </si>
+  <si>
+    <t>Include units in column names</t>
+  </si>
+  <si>
+    <t>Einheiten in Spaltennamen aufnehmen</t>
+  </si>
+  <si>
+    <t>Localize column names</t>
+  </si>
+  <si>
+    <t>Output file</t>
+  </si>
+  <si>
+    <t>Excel Files (*.xlsx)</t>
+  </si>
+  <si>
+    <t>Please select at last one impact.</t>
+  </si>
+  <si>
+    <t>Please chose an .xlsx file.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excel export finished </t>
+  </si>
+  <si>
+    <t>Failed to export Excel</t>
+  </si>
+  <si>
+    <t>Fehler beim Excel-Export</t>
+  </si>
+  <si>
+    <t>Excel-Export abgeschlossen</t>
+  </si>
+  <si>
+    <t>Bitte eine .xlsx-Datei wählen.</t>
+  </si>
+  <si>
+    <t>Bitte mindestens einen Impact auswählen.</t>
+  </si>
+  <si>
+    <t>Excel-Dateien (*.xlsx)</t>
+  </si>
+  <si>
+    <t>Ausgabedatei</t>
+  </si>
+  <si>
+    <t>Spaltennamen lokalisieren</t>
   </si>
 </sst>
 </file>
@@ -2445,7 +2520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J167"/>
+  <dimension ref="A1:J177"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="60.5703125" style="4" customWidth="1"/>
@@ -3798,6 +3873,86 @@
         <v>376</v>
       </c>
     </row>
+    <row r="168" spans="1:2" ht="15" customHeight="1">
+      <c r="A168" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" ht="15" customHeight="1">
+      <c r="A169" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="B169" s="7" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" ht="15" customHeight="1">
+      <c r="A170" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="B170" s="7" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" ht="15" customHeight="1">
+      <c r="A171" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="B171" s="4" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" ht="15" customHeight="1">
+      <c r="A172" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="B172" s="7" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" ht="15" customHeight="1">
+      <c r="A173" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="B173" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" ht="15" customHeight="1">
+      <c r="A174" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="B174" s="7" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" ht="15" customHeight="1">
+      <c r="A175" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="B175" s="7" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" ht="15" customHeight="1">
+      <c r="A176" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="B176" s="7" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" ht="15" customHeight="1">
+      <c r="A177" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="B177" s="7" t="s">
+        <v>395</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
@@ -3809,7 +3964,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B168"/>
+  <dimension ref="A1:B180"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="54.140625" style="4" customWidth="1"/>
@@ -4983,7 +5138,7 @@
         <v>282</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>283</v>
+        <v>379</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="15" customHeight="1">
@@ -4991,7 +5146,7 @@
         <v>284</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>285</v>
+        <v>380</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="15" customHeight="1">
@@ -5160,6 +5315,102 @@
       </c>
       <c r="B168" s="7" t="s">
         <v>377</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" ht="15" customHeight="1">
+      <c r="A169" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" ht="15" customHeight="1">
+      <c r="A170" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="B170" s="7" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" ht="15" customHeight="1">
+      <c r="A171" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="B171" s="7" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" ht="15" customHeight="1">
+      <c r="A172" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="B172" s="7" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" ht="15" customHeight="1">
+      <c r="A173" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="B173" s="4" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" ht="15" customHeight="1">
+      <c r="A174" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="B174" s="4" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" ht="15" customHeight="1">
+      <c r="A175" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="B175" s="4" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" ht="15" customHeight="1">
+      <c r="A176" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="B176" s="4" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" ht="15" customHeight="1">
+      <c r="A177" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="B177" s="7" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" ht="15" customHeight="1">
+      <c r="A178" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="B178" s="4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" ht="15" customHeight="1">
+      <c r="A179" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="B179" s="4" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" ht="15" customHeight="1">
+      <c r="A180" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="B180" s="4" t="s">
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -5173,11 +5424,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B171"/>
+  <dimension ref="A1:B181"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="64" style="4" customWidth="1"/>
-    <col min="2" max="2" width="49.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="115" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="9.140625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -6548,6 +6799,86 @@
       </c>
       <c r="B171" s="7" t="s">
         <v>376</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" ht="15" customHeight="1">
+      <c r="A172" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="B172" s="4" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" ht="15" customHeight="1">
+      <c r="A173" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="B173" s="7" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" ht="15" customHeight="1">
+      <c r="A174" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="B174" s="7" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" ht="15" customHeight="1">
+      <c r="A175" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="B175" s="4" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" ht="15" customHeight="1">
+      <c r="A176" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="B176" s="7" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" ht="15" customHeight="1">
+      <c r="A177" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="B177" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" ht="15" customHeight="1">
+      <c r="A178" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="B178" s="7" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" ht="15" customHeight="1">
+      <c r="A179" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="B179" s="7" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" ht="15" customHeight="1">
+      <c r="A180" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="B180" s="7" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" ht="15" customHeight="1">
+      <c r="A181" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="B181" s="7" t="s">
+        <v>395</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Export to Excel function
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59270F15-0AB1-49CD-A204-08B043228A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D52434-DA18-4CC0-8CE1-8FAF5005BA41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="404">
   <si>
     <t>exiobase</t>
   </si>
@@ -1184,9 +1184,6 @@
     <t>Aktualisieren</t>
   </si>
   <si>
-    <t>Daten exportieren</t>
-  </si>
-  <si>
     <t>Impacts</t>
   </si>
   <si>
@@ -1196,9 +1193,6 @@
     <t>Einheiten in Spaltennamen aufnehmen</t>
   </si>
   <si>
-    <t>Localize column names</t>
-  </si>
-  <si>
     <t>Output file</t>
   </si>
   <si>
@@ -1235,7 +1229,16 @@
     <t>Ausgabedatei</t>
   </si>
   <si>
-    <t>Spaltennamen lokalisieren</t>
+    <t>Choose impacts</t>
+  </si>
+  <si>
+    <t>Wähle Impacts aus</t>
+  </si>
+  <si>
+    <t>Excel export finished</t>
+  </si>
+  <si>
+    <t>Daten exportieren (Excel)</t>
   </si>
 </sst>
 </file>
@@ -2524,7 +2527,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="60.5703125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="41.7109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="115" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="9.140625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -3883,74 +3886,74 @@
     </row>
     <row r="169" spans="1:2" ht="15" customHeight="1">
       <c r="A169" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B169" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="15" customHeight="1">
       <c r="A170" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B170" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="15" customHeight="1">
-      <c r="A171" s="4" t="s">
-        <v>389</v>
-      </c>
-      <c r="B171" s="4" t="s">
-        <v>389</v>
+      <c r="A171" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="B171" s="7" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="15" customHeight="1">
       <c r="A172" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B172" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="15" customHeight="1">
       <c r="A173" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B173" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="174" spans="1:2" ht="15" customHeight="1">
       <c r="A174" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B174" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="15" customHeight="1">
       <c r="A175" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B175" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="15" customHeight="1">
       <c r="A176" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B176" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="15" customHeight="1">
       <c r="A177" s="7" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="B177" s="7" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -5338,79 +5341,79 @@
         <v>383</v>
       </c>
       <c r="B171" s="7" t="s">
-        <v>385</v>
+        <v>403</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="15" customHeight="1">
       <c r="A172" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B172" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="15" customHeight="1">
       <c r="A173" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="B173" s="4" t="s">
         <v>387</v>
       </c>
-      <c r="B173" s="4" t="s">
+    </row>
+    <row r="174" spans="1:2" ht="15" customHeight="1">
+      <c r="A174" s="7" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="174" spans="1:2" ht="15" customHeight="1">
-      <c r="A174" s="4" t="s">
-        <v>389</v>
-      </c>
       <c r="B174" s="4" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="15" customHeight="1">
       <c r="A175" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="15" customHeight="1">
       <c r="A176" s="7" t="s">
-        <v>391</v>
-      </c>
-      <c r="B176" s="4" t="s">
-        <v>400</v>
+        <v>390</v>
+      </c>
+      <c r="B176" s="7" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="15" customHeight="1">
       <c r="A177" s="7" t="s">
-        <v>392</v>
-      </c>
-      <c r="B177" s="7" t="s">
-        <v>399</v>
+        <v>391</v>
+      </c>
+      <c r="B177" s="4" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="15" customHeight="1">
       <c r="A178" s="7" t="s">
-        <v>393</v>
+        <v>402</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="179" spans="1:2" ht="15" customHeight="1">
       <c r="A179" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="B179" s="4" t="s">
         <v>394</v>
-      </c>
-      <c r="B179" s="4" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="15" customHeight="1">
       <c r="A180" s="7" t="s">
-        <v>395</v>
-      </c>
-      <c r="B180" s="4" t="s">
-        <v>396</v>
+        <v>400</v>
+      </c>
+      <c r="B180" s="7" t="s">
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -6811,74 +6814,74 @@
     </row>
     <row r="173" spans="1:2" ht="15" customHeight="1">
       <c r="A173" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B173" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="174" spans="1:2" ht="15" customHeight="1">
       <c r="A174" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B174" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="15" customHeight="1">
-      <c r="A175" s="4" t="s">
-        <v>389</v>
-      </c>
-      <c r="B175" s="4" t="s">
-        <v>389</v>
+      <c r="A175" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="B175" s="7" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="15" customHeight="1">
       <c r="A176" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B176" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="15" customHeight="1">
       <c r="A177" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B177" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="15" customHeight="1">
       <c r="A178" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B178" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="179" spans="1:2" ht="15" customHeight="1">
       <c r="A179" s="7" t="s">
-        <v>393</v>
+        <v>402</v>
       </c>
       <c r="B179" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="15" customHeight="1">
       <c r="A180" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B180" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="181" spans="1:2" ht="15" customHeight="1">
       <c r="A181" s="7" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="B181" s="7" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Provided information about parameters in the advanced settings
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D52434-DA18-4CC0-8CE1-8FAF5005BA41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D852A82-52E2-4100-9C52-494C83ABE1B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="471">
   <si>
     <t>exiobase</t>
   </si>
@@ -500,9 +500,6 @@
     <t>Klassen (k)</t>
   </si>
   <si>
-    <t>Costum bins (kommagetrennt)</t>
-  </si>
-  <si>
     <t>Normalisierung (fließender Modus)</t>
   </si>
   <si>
@@ -1239,17 +1236,240 @@
   </si>
   <si>
     <t>Daten exportieren (Excel)</t>
+  </si>
+  <si>
+    <t>Continuous: Colors and legend use absolute values. Use Norm + Robust clipping + Gamma to control contrast.</t>
+  </si>
+  <si>
+    <t>Continuous: Farben und Legende basieren auf absoluten Werten. Kontrast über Normierung + Robustes Clipping + Gamma steuern.</t>
+  </si>
+  <si>
+    <t>Binned: Diskrete Klassen. Mit „Relativ“ klassifizierst Du nach Prozentanteilen (Summe = 100 %); sonst nach absoluten Werten.</t>
+  </si>
+  <si>
+    <t>Binned: Discrete classes. With 'Relative' you classify by percentage shares (sum = 100%); otherwise by absolute values.</t>
+  </si>
+  <si>
+    <t>Appearance</t>
+  </si>
+  <si>
+    <t>Darstellung</t>
+  </si>
+  <si>
+    <t>Binning (binned mode)</t>
+  </si>
+  <si>
+    <t>Klasseneinteilung (binned)</t>
+  </si>
+  <si>
+    <t>Relative</t>
+  </si>
+  <si>
+    <t>Relativ</t>
+  </si>
+  <si>
+    <t>Eigene Klassen (kommagetrennt)</t>
+  </si>
+  <si>
+    <t>Continuous scaling</t>
+  </si>
+  <si>
+    <t>Normierung</t>
+  </si>
+  <si>
+    <t>Robustes Clipping (%)</t>
+  </si>
+  <si>
+    <t>Gamma (Power-Norm)</t>
+  </si>
+  <si>
+    <t>Choose a color palette for the map.</t>
+  </si>
+  <si>
+    <t>Wähle eine Farbpalette für die Karte.</t>
+  </si>
+  <si>
+    <t>Invert the colormap.</t>
+  </si>
+  <si>
+    <t>Kehrt die Farbpalette um.</t>
+  </si>
+  <si>
+    <t>Show colorbar with value ranges.</t>
+  </si>
+  <si>
+    <t>Zeigt die Farbskala mit Wertebereichen an.</t>
+  </si>
+  <si>
+    <t>Optional title displayed above the map.</t>
+  </si>
+  <si>
+    <t>Optionaler Titel oberhalb der Karte.</t>
+  </si>
+  <si>
+    <t>Choose between binned (discrete classes) or continuous scale.</t>
+  </si>
+  <si>
+    <t>If checked, classes use percentage shares (sum=100%). If unchecked, absolute values.</t>
+  </si>
+  <si>
+    <t>Wenn aktiv, werden Klassen nach Anteilen in Prozent (Summe=100 %) gebildet; sonst nach absoluten Werten.</t>
+  </si>
+  <si>
+    <t>Number of classes when no custom bins are provided.</t>
+  </si>
+  <si>
+    <t>Anzahl der Klassen, wenn keine eigenen Grenzen angegeben sind.</t>
+  </si>
+  <si>
+    <t>Comma-separated inner class boundaries. dmin and dmax are added automatically.</t>
+  </si>
+  <si>
+    <t>Kommagetrennte innere Klassengrenzen. Minimum und Maximum werden automatisch ergänzt.</t>
+  </si>
+  <si>
+    <t>Quantile clipping for vmin/vmax (e.g., 2% uses 2nd and 98th percentiles).</t>
+  </si>
+  <si>
+    <t>Bestimmt vmin/vmax über Quantile (z. B. 2 % nutzt 2. und 98. Perzentil).</t>
+  </si>
+  <si>
+    <t>PowerNorm exponent: &lt;1 enhances small values, &gt;1 enhances large values.</t>
+  </si>
+  <si>
+    <t>Exponent für PowerNorm: &lt;1 betont kleine Werte, &gt;1 betont große Werte.</t>
+  </si>
+  <si>
+    <t>Colormap used to color the countries. Use 'Reverse' to invert light/dark order.</t>
+  </si>
+  <si>
+    <t>Farbpalette zur Einfärbung der Länder. Mit „Umkehren“ wird die Hell/Dunkel-Reihenfolge invertiert.</t>
+  </si>
+  <si>
+    <t>Inverts the selected colormap.</t>
+  </si>
+  <si>
+    <t>Invertiert die gewählte Farbpalette.</t>
+  </si>
+  <si>
+    <t>Displays a legend. In continuous mode it shows absolute values; in binned mode it shows numeric ranges per class.</t>
+  </si>
+  <si>
+    <t>Blendet eine Legende ein. Im Modus „continuous“ zeigt sie absolute Werte, im Modus „binned“ numerische Klassenbereiche.</t>
+  </si>
+  <si>
+    <t>Optional title for the map.</t>
+  </si>
+  <si>
+    <t>Optionaler Titel für die Karte.</t>
+  </si>
+  <si>
+    <t>continuous: Colors reflect absolute values with a continuous legend.
+binned: Discrete classes. With 'Relative' you bin by percentage shares.</t>
+  </si>
+  <si>
+    <t>continuous: Farben spiegeln absolute Werte wider, die Legende ist stetig.
+binned: Diskrete Klassen. Mit „Relativ“ erfolgt die Einteilung nach Prozentanteilen.</t>
+  </si>
+  <si>
+    <t>Binned mode only: toggle between absolute values and percentage shares for the class breaks.</t>
+  </si>
+  <si>
+    <t>Nur im binned-Modus: Umschalten zwischen absoluten Werten und Prozentanteilen für die Klassengrenzen.</t>
+  </si>
+  <si>
+    <t>Number of discrete classes. If 'Custom bins' are provided, they take precedence.</t>
+  </si>
+  <si>
+    <t>Anzahl der diskreten Klassen. Bei „Eigene Klassen“ haben diese Vorrang.</t>
+  </si>
+  <si>
+    <t>Enter inner edges like '10, 25, 50'. The dialog will prepend the data minimum and append the maximum.</t>
+  </si>
+  <si>
+    <t>Innere Kanten eingeben, z. B. „10, 25, 50“. Minimum und Maximum werden automatisch ergänzt.</t>
+  </si>
+  <si>
+    <t>Normalization for continuous mode:
+- linear: uniform mapping from vmin..vmax
+- log: logarithmic mapping; requires strictly positive values
+- power: Power-law mapping; see Gamma</t>
+  </si>
+  <si>
+    <t>Normierung für den continuous-Modus:
+- linear: gleichmäßige Abbildung von vmin..vmax
+- log: logarithmische Abbildung; nur für strikt positive Werte
+- power: Potenz-Abbildung; siehe Gamma</t>
+  </si>
+  <si>
+    <t>Robust clipping determines vmin/vmax from quantiles instead of absolute min/max to reduce outlier effects.</t>
+  </si>
+  <si>
+    <t>Robustes Clipping bestimmt vmin/vmax über Quantile statt über Min/Max, um Ausreißer zu dämpfen.</t>
+  </si>
+  <si>
+    <t>Gamma (PowerNorm):
+- gamma &lt; 1 emphasises lower value range
+- gamma &gt; 1 emphasises higher value range</t>
+  </si>
+  <si>
+    <t>Gamma (PowerNorm):
+- gamma &lt; 1 betont den unteren Wertebereich
+- gamma &gt; 1 betont den oberen Wertebereich</t>
+  </si>
+  <si>
+    <t>Linear: uniform color steps from vmin to vmax.</t>
+  </si>
+  <si>
+    <t>Linear: gleichmäßige Farbabstufung von vmin bis vmax.</t>
+  </si>
+  <si>
+    <t>Log: emphasises orders of magnitude; requires strictly positive data.</t>
+  </si>
+  <si>
+    <t>Log: betont Größenordnungen; erfordert strikt positive Daten.</t>
+  </si>
+  <si>
+    <t>Power: adjust contrast with Gamma (&lt;1: highlights small values; &gt;1: highlights large).</t>
+  </si>
+  <si>
+    <t>Power: Kontrast über Gamma steuern (&lt;1: betont kleine Werte; &gt;1: betont große).</t>
+  </si>
+  <si>
+    <t>Help</t>
+  </si>
+  <si>
+    <t>Hilfe</t>
+  </si>
+  <si>
+    <t>Wähle zwischen diskreten Klassen (binned) und stetiger Skala (continuous).</t>
+  </si>
+  <si>
+    <t>linear: uniform steps | log: highlight orders of magnitude (logarithmic) | power: adjustable contrast with gamma</t>
+  </si>
+  <si>
+    <t>linear: gleichmäßige Schritte | log: betont Größenordnungen (logarithmisch) | power: anpassbarer Kontrast mit Gamma</t>
+  </si>
+  <si>
+    <t>Stetige Skalierung (continuous)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1340,32 +1560,34 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="1" xr:uid="{C2F78208-F7F8-4542-9E5B-6270DCB86735}"/>
+    <cellStyle name="Standard 3" xfId="2" xr:uid="{C71F7E32-9819-48E7-8142-C8147DEC96B1}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
@@ -3214,58 +3436,58 @@
     </row>
     <row r="85" spans="1:2" ht="15" customHeight="1">
       <c r="A85" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="15" customHeight="1">
       <c r="A86" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="15" customHeight="1">
       <c r="A87" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="15" customHeight="1">
       <c r="A88" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="15" customHeight="1">
       <c r="A89" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="15" customHeight="1">
       <c r="A90" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="15" customHeight="1">
       <c r="A91" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="15" customHeight="1">
@@ -3278,682 +3500,682 @@
     </row>
     <row r="93" spans="1:2" ht="15" customHeight="1">
       <c r="A93" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="15" customHeight="1">
       <c r="A94" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="15" customHeight="1">
       <c r="A95" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="15" customHeight="1">
       <c r="A96" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="15" customHeight="1">
       <c r="A97" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="15" customHeight="1">
       <c r="A98" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="15" customHeight="1">
       <c r="A99" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="15" customHeight="1">
       <c r="A100" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="15" customHeight="1">
       <c r="A101" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="15" customHeight="1">
       <c r="A102" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="15" customHeight="1">
       <c r="A103" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="15" customHeight="1">
       <c r="A104" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="105" spans="1:2" ht="15" customHeight="1">
       <c r="A105" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="15" customHeight="1">
       <c r="A106" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="15" customHeight="1">
       <c r="A107" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="15" customHeight="1">
       <c r="A108" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="15" customHeight="1">
       <c r="A109" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="110" spans="1:2" ht="15" customHeight="1">
       <c r="A110" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="15" customHeight="1">
       <c r="A111" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="15" customHeight="1">
       <c r="A112" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="113" spans="1:2" ht="15" customHeight="1">
       <c r="A113" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="15" customHeight="1">
       <c r="A114" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="15" customHeight="1">
       <c r="A115" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="15" customHeight="1">
       <c r="A116" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="15" customHeight="1">
       <c r="A117" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="15" customHeight="1">
       <c r="A118" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="15" customHeight="1">
       <c r="A119" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="120" spans="1:2" ht="15" customHeight="1">
       <c r="A120" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="15" customHeight="1">
       <c r="A121" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="15" customHeight="1">
       <c r="A122" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="15" customHeight="1">
       <c r="A123" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="15" customHeight="1">
       <c r="A124" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="125" spans="1:2" ht="15" customHeight="1">
       <c r="A125" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="126" spans="1:2" ht="15" customHeight="1">
       <c r="A126" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="15" customHeight="1">
       <c r="A127" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="15" customHeight="1">
       <c r="A128" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="15" customHeight="1">
       <c r="A129" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="15" customHeight="1">
       <c r="A130" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="15" customHeight="1">
       <c r="A131" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="15" customHeight="1">
       <c r="A132" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="15" customHeight="1">
       <c r="A133" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="15" customHeight="1">
       <c r="A134" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="15" customHeight="1">
       <c r="A135" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="15" customHeight="1">
       <c r="A136" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="137" spans="1:2" ht="15" customHeight="1">
       <c r="A137" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="15" customHeight="1">
       <c r="A138" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="15" customHeight="1">
       <c r="A139" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="15" customHeight="1">
       <c r="A140" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="15" customHeight="1">
       <c r="A141" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B141" s="4" t="s">
         <v>272</v>
-      </c>
-      <c r="B141" s="4" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="15" customHeight="1">
       <c r="A142" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B142" s="4" t="s">
         <v>274</v>
-      </c>
-      <c r="B142" s="4" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="15" customHeight="1">
       <c r="A143" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B143" s="4" t="s">
         <v>276</v>
-      </c>
-      <c r="B143" s="4" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="15" customHeight="1">
       <c r="A144" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B144" s="4" t="s">
         <v>278</v>
-      </c>
-      <c r="B144" s="4" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="15" customHeight="1">
       <c r="A145" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B145" s="4" t="s">
         <v>280</v>
-      </c>
-      <c r="B145" s="4" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="15" customHeight="1">
       <c r="A146" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B146" s="4" t="s">
         <v>282</v>
-      </c>
-      <c r="B146" s="4" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="15" customHeight="1">
       <c r="A147" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B147" s="4" t="s">
         <v>284</v>
-      </c>
-      <c r="B147" s="4" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="15" customHeight="1">
       <c r="A148" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B148" s="4" t="s">
         <v>286</v>
-      </c>
-      <c r="B148" s="4" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="15" customHeight="1">
       <c r="A149" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B149" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="15" customHeight="1">
       <c r="A150" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B150" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="15" customHeight="1">
       <c r="A151" s="7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B151" s="7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="15" customHeight="1">
       <c r="A152" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B152" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="15" customHeight="1">
       <c r="A153" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B153" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="15" customHeight="1">
       <c r="A154" s="7" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B154" s="7" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="15" customHeight="1">
       <c r="A155" s="7" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B155" s="7" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="15" customHeight="1">
       <c r="A156" s="7" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B156" s="7" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="157" spans="1:2" ht="15" customHeight="1">
       <c r="A157" s="7" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B157" s="7" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="15" customHeight="1">
       <c r="A158" s="7" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B158" s="7" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="15" customHeight="1">
       <c r="A159" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="160" spans="1:2" ht="15" customHeight="1">
       <c r="A160" s="7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B160" s="7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="161" spans="1:2" ht="15" customHeight="1">
       <c r="A161" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B161" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="162" spans="1:2" ht="15" customHeight="1">
       <c r="A162" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B162" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="15" customHeight="1">
       <c r="A163" s="7" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B163" s="7" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="164" spans="1:2" ht="15" customHeight="1">
       <c r="A164" s="7" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B164" s="7" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="165" spans="1:2" ht="15" customHeight="1">
       <c r="A165" s="7" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B165" s="7" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="15" customHeight="1">
       <c r="A166" s="7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B166" s="7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="15" customHeight="1">
       <c r="A167" s="7" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B167" s="7" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="168" spans="1:2" ht="15" customHeight="1">
       <c r="A168" s="4" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="15" customHeight="1">
       <c r="A169" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B169" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="15" customHeight="1">
       <c r="A170" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B170" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="15" customHeight="1">
       <c r="A171" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B171" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="15" customHeight="1">
       <c r="A172" s="7" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B172" s="7" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="15" customHeight="1">
       <c r="A173" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B173" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="174" spans="1:2" ht="15" customHeight="1">
       <c r="A174" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B174" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="15" customHeight="1">
       <c r="A175" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B175" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="15" customHeight="1">
       <c r="A176" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B176" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="15" customHeight="1">
       <c r="A177" s="7" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B177" s="7" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
   </sheetData>
@@ -3967,11 +4189,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B180"/>
+  <dimension ref="A1:B213"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="54.140625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="54.28515625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="67" style="4" customWidth="1"/>
+    <col min="2" max="2" width="62" style="4" customWidth="1"/>
     <col min="3" max="6" width="9.140625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -4541,7 +4763,7 @@
         <v>138</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="15" customHeight="1">
@@ -4589,7 +4811,7 @@
         <v>144</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>157</v>
+        <v>413</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="15" customHeight="1">
@@ -4597,7 +4819,7 @@
         <v>145</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="15" customHeight="1">
@@ -4621,7 +4843,7 @@
         <v>148</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="15" customHeight="1">
@@ -4629,7 +4851,7 @@
         <v>149</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="15" customHeight="1">
@@ -4637,7 +4859,7 @@
         <v>150</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>150</v>
+        <v>416</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="15" customHeight="1">
@@ -4645,63 +4867,63 @@
         <v>151</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>151</v>
+        <v>417</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="15" customHeight="1">
       <c r="A85" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="15" customHeight="1">
       <c r="A86" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="15" customHeight="1">
       <c r="A87" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="15" customHeight="1">
       <c r="A88" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="15" customHeight="1">
       <c r="A89" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="15" customHeight="1">
       <c r="A90" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="15" customHeight="1">
       <c r="A91" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B91" s="4" t="s">
         <v>174</v>
-      </c>
-      <c r="B91" s="4" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="15" customHeight="1">
@@ -4709,711 +4931,975 @@
         <v>135</v>
       </c>
       <c r="B92" s="7" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="15" customHeight="1">
       <c r="A93" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B93" s="4" t="s">
         <v>176</v>
-      </c>
-      <c r="B93" s="4" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="15" customHeight="1">
       <c r="A94" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B94" s="4" t="s">
         <v>178</v>
-      </c>
-      <c r="B94" s="4" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="15" customHeight="1">
       <c r="A95" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B95" s="4" t="s">
         <v>180</v>
-      </c>
-      <c r="B95" s="4" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="15" customHeight="1">
       <c r="A96" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B96" s="4" t="s">
         <v>182</v>
-      </c>
-      <c r="B96" s="4" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="15" customHeight="1">
       <c r="A97" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B97" s="4" t="s">
         <v>184</v>
-      </c>
-      <c r="B97" s="4" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="15" customHeight="1">
       <c r="A98" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B98" s="4" t="s">
         <v>186</v>
-      </c>
-      <c r="B98" s="4" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="15" customHeight="1">
       <c r="A99" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B99" s="4" t="s">
         <v>188</v>
-      </c>
-      <c r="B99" s="4" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="15" customHeight="1">
       <c r="A100" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B100" s="4" t="s">
         <v>190</v>
-      </c>
-      <c r="B100" s="4" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="15" customHeight="1">
       <c r="A101" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B101" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="B101" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="15" customHeight="1">
       <c r="A102" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B102" s="4" t="s">
         <v>194</v>
-      </c>
-      <c r="B102" s="4" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="15" customHeight="1">
       <c r="A103" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B103" s="4" t="s">
         <v>196</v>
-      </c>
-      <c r="B103" s="4" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="15" customHeight="1">
       <c r="A104" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B104" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="B104" s="4" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="105" spans="1:2" ht="15" customHeight="1">
       <c r="A105" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B105" s="4" t="s">
         <v>200</v>
-      </c>
-      <c r="B105" s="4" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="15" customHeight="1">
       <c r="A106" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B106" s="4" t="s">
         <v>202</v>
-      </c>
-      <c r="B106" s="4" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="15" customHeight="1">
       <c r="A107" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B107" s="4" t="s">
         <v>204</v>
-      </c>
-      <c r="B107" s="4" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="15" customHeight="1">
       <c r="A108" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B108" s="4" t="s">
         <v>206</v>
-      </c>
-      <c r="B108" s="4" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="15" customHeight="1">
       <c r="A109" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B109" s="4" t="s">
         <v>208</v>
-      </c>
-      <c r="B109" s="4" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="110" spans="1:2" ht="15" customHeight="1">
       <c r="A110" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B110" s="4" t="s">
         <v>210</v>
-      </c>
-      <c r="B110" s="4" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="15" customHeight="1">
       <c r="A111" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B111" s="4" t="s">
         <v>212</v>
-      </c>
-      <c r="B111" s="4" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="15" customHeight="1">
       <c r="A112" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B112" s="4" t="s">
         <v>214</v>
-      </c>
-      <c r="B112" s="4" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="113" spans="1:2" ht="15" customHeight="1">
       <c r="A113" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B113" s="4" t="s">
         <v>216</v>
-      </c>
-      <c r="B113" s="4" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="15" customHeight="1">
       <c r="A114" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B114" s="4" t="s">
         <v>218</v>
-      </c>
-      <c r="B114" s="4" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="15" customHeight="1">
       <c r="A115" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B115" s="4" t="s">
         <v>220</v>
-      </c>
-      <c r="B115" s="4" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="15" customHeight="1">
       <c r="A116" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B116" s="4" t="s">
         <v>222</v>
-      </c>
-      <c r="B116" s="4" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="15" customHeight="1">
       <c r="A117" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B117" s="4" t="s">
         <v>224</v>
-      </c>
-      <c r="B117" s="4" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="15" customHeight="1">
       <c r="A118" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B118" s="4" t="s">
         <v>226</v>
-      </c>
-      <c r="B118" s="4" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="15" customHeight="1">
       <c r="A119" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B119" s="4" t="s">
         <v>228</v>
-      </c>
-      <c r="B119" s="4" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="120" spans="1:2" ht="15" customHeight="1">
       <c r="A120" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B120" s="4" t="s">
         <v>230</v>
-      </c>
-      <c r="B120" s="4" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="15" customHeight="1">
       <c r="A121" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B121" s="4" t="s">
         <v>232</v>
-      </c>
-      <c r="B121" s="4" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="15" customHeight="1">
       <c r="A122" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B122" s="4" t="s">
         <v>234</v>
-      </c>
-      <c r="B122" s="4" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="15" customHeight="1">
       <c r="A123" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B123" s="4" t="s">
         <v>236</v>
-      </c>
-      <c r="B123" s="4" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="15" customHeight="1">
       <c r="A124" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B124" s="4" t="s">
         <v>238</v>
-      </c>
-      <c r="B124" s="4" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="125" spans="1:2" ht="15" customHeight="1">
       <c r="A125" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B125" s="4" t="s">
         <v>240</v>
-      </c>
-      <c r="B125" s="4" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="126" spans="1:2" ht="15" customHeight="1">
       <c r="A126" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B126" s="4" t="s">
         <v>242</v>
-      </c>
-      <c r="B126" s="4" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="15" customHeight="1">
       <c r="A127" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B127" s="4" t="s">
         <v>244</v>
-      </c>
-      <c r="B127" s="4" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="15" customHeight="1">
       <c r="A128" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B128" s="4" t="s">
         <v>246</v>
-      </c>
-      <c r="B128" s="4" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="15" customHeight="1">
       <c r="A129" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B129" s="4" t="s">
         <v>248</v>
-      </c>
-      <c r="B129" s="4" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="15" customHeight="1">
       <c r="A130" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B130" s="4" t="s">
         <v>250</v>
-      </c>
-      <c r="B130" s="4" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="15" customHeight="1">
       <c r="A131" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B131" s="4" t="s">
         <v>252</v>
-      </c>
-      <c r="B131" s="4" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="15" customHeight="1">
       <c r="A132" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="B132" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="B132" s="4" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="15" customHeight="1">
       <c r="A133" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B133" s="4" t="s">
         <v>256</v>
-      </c>
-      <c r="B133" s="4" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="15" customHeight="1">
       <c r="A134" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="B134" s="4" t="s">
         <v>258</v>
-      </c>
-      <c r="B134" s="4" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="15" customHeight="1">
       <c r="A135" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B135" s="4" t="s">
         <v>260</v>
-      </c>
-      <c r="B135" s="4" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="15" customHeight="1">
       <c r="A136" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B136" s="4" t="s">
         <v>262</v>
-      </c>
-      <c r="B136" s="4" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="137" spans="1:2" ht="15" customHeight="1">
       <c r="A137" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B137" s="4" t="s">
         <v>264</v>
-      </c>
-      <c r="B137" s="4" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="15" customHeight="1">
       <c r="A138" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="B138" s="4" t="s">
         <v>266</v>
-      </c>
-      <c r="B138" s="4" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="15" customHeight="1">
       <c r="A139" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B139" s="4" t="s">
         <v>268</v>
-      </c>
-      <c r="B139" s="4" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="15" customHeight="1">
       <c r="A140" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B140" s="4" t="s">
         <v>270</v>
-      </c>
-      <c r="B140" s="4" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="15" customHeight="1">
       <c r="A141" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B141" s="4" t="s">
         <v>272</v>
-      </c>
-      <c r="B141" s="4" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="15" customHeight="1">
       <c r="A142" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B142" s="4" t="s">
         <v>274</v>
-      </c>
-      <c r="B142" s="4" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="15" customHeight="1">
       <c r="A143" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B143" s="4" t="s">
         <v>276</v>
-      </c>
-      <c r="B143" s="4" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="15" customHeight="1">
       <c r="A144" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B144" s="4" t="s">
         <v>278</v>
-      </c>
-      <c r="B144" s="4" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="15" customHeight="1">
       <c r="A145" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B145" s="4" t="s">
         <v>280</v>
-      </c>
-      <c r="B145" s="4" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="15" customHeight="1">
       <c r="A146" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="15" customHeight="1">
       <c r="A147" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="15" customHeight="1">
       <c r="A148" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B148" s="4" t="s">
         <v>286</v>
-      </c>
-      <c r="B148" s="4" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="15" customHeight="1">
       <c r="A149" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="B149" s="7" t="s">
         <v>337</v>
-      </c>
-      <c r="B149" s="7" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="15" customHeight="1">
       <c r="A150" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B150" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="15" customHeight="1">
       <c r="A151" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="B151" s="7" t="s">
         <v>340</v>
-      </c>
-      <c r="B151" s="7" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="15" customHeight="1">
       <c r="A152" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B152" s="7" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="15" customHeight="1">
       <c r="A153" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="B153" s="7" t="s">
         <v>344</v>
-      </c>
-      <c r="B153" s="7" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="15" customHeight="1">
       <c r="A154" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="B154" s="7" t="s">
         <v>346</v>
-      </c>
-      <c r="B154" s="7" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="15" customHeight="1">
       <c r="A155" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="B155" s="7" t="s">
         <v>348</v>
-      </c>
-      <c r="B155" s="7" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="15" customHeight="1">
       <c r="A156" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="B156" s="7" t="s">
         <v>350</v>
-      </c>
-      <c r="B156" s="7" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="157" spans="1:2" ht="15" customHeight="1">
       <c r="A157" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="B157" s="7" t="s">
         <v>352</v>
-      </c>
-      <c r="B157" s="7" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="15" customHeight="1">
       <c r="A158" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="B158" s="7" t="s">
         <v>354</v>
-      </c>
-      <c r="B158" s="7" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="15" customHeight="1">
       <c r="A159" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="B159" s="7" t="s">
         <v>357</v>
-      </c>
-      <c r="B159" s="7" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="160" spans="1:2" ht="15" customHeight="1">
       <c r="A160" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B160" s="7" t="s">
         <v>359</v>
-      </c>
-      <c r="B160" s="7" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="161" spans="1:2" ht="15" customHeight="1">
       <c r="A161" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="B161" s="7" t="s">
         <v>361</v>
-      </c>
-      <c r="B161" s="7" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="162" spans="1:2" ht="15" customHeight="1">
       <c r="A162" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B162" s="7" t="s">
         <v>363</v>
-      </c>
-      <c r="B162" s="7" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="15" customHeight="1">
       <c r="A163" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="B163" s="7" t="s">
         <v>365</v>
-      </c>
-      <c r="B163" s="7" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="164" spans="1:2" ht="15" customHeight="1">
       <c r="A164" s="7" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B164" s="7" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="165" spans="1:2" ht="15" customHeight="1">
       <c r="A165" s="7" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B165" s="7" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="15" customHeight="1">
       <c r="A166" s="7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B166" s="7" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="15" customHeight="1">
       <c r="A167" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="B167" s="7" t="s">
         <v>374</v>
-      </c>
-      <c r="B167" s="7" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="168" spans="1:2" ht="15" customHeight="1">
       <c r="A168" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="B168" s="7" t="s">
         <v>376</v>
-      </c>
-      <c r="B168" s="7" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="15" customHeight="1">
       <c r="A169" s="4" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="15" customHeight="1">
       <c r="A170" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B170" s="7" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="15" customHeight="1">
       <c r="A171" s="7" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B171" s="7" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="15" customHeight="1">
       <c r="A172" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B172" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="15" customHeight="1">
       <c r="A173" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="B173" s="4" t="s">
         <v>386</v>
-      </c>
-      <c r="B173" s="4" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="174" spans="1:2" ht="15" customHeight="1">
       <c r="A174" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="15" customHeight="1">
       <c r="A175" s="7" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="15" customHeight="1">
       <c r="A176" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B176" s="7" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="15" customHeight="1">
       <c r="A177" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="15" customHeight="1">
       <c r="A178" s="7" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="179" spans="1:2" ht="15" customHeight="1">
       <c r="A179" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="B179" s="4" t="s">
         <v>393</v>
-      </c>
-      <c r="B179" s="4" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="15" customHeight="1">
       <c r="A180" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="B180" s="7" t="s">
         <v>400</v>
       </c>
-      <c r="B180" s="7" t="s">
-        <v>401</v>
+    </row>
+    <row r="181" spans="1:2" ht="15" customHeight="1">
+      <c r="A181" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="B181" s="4" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" ht="15" customHeight="1">
+      <c r="A182" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="B182" s="4" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" ht="15" customHeight="1">
+      <c r="A183" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="B183" s="4" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" ht="15" customHeight="1">
+      <c r="A184" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="B184" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" ht="15" customHeight="1">
+      <c r="A185" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="B185" s="7" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" ht="15" customHeight="1">
+      <c r="A186" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="B186" s="4" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" ht="15" customHeight="1">
+      <c r="A187" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B187" s="4" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" ht="15" customHeight="1">
+      <c r="A188" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="B188" s="4" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" ht="15" customHeight="1">
+      <c r="A189" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="B189" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" ht="15" customHeight="1">
+      <c r="A190" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="B190" s="4" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" ht="15" customHeight="1">
+      <c r="A191" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="B191" s="4" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" ht="15" customHeight="1">
+      <c r="A192" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="B192" s="4" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" ht="15" customHeight="1">
+      <c r="A193" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="B193" s="4" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" ht="15" customHeight="1">
+      <c r="A194" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="B194" s="4" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" ht="15" customHeight="1">
+      <c r="A195" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="B195" s="4" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" ht="15" customHeight="1">
+      <c r="A196" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="B196" s="4" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" ht="15" customHeight="1">
+      <c r="A197" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="B197" s="4" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" ht="15" customHeight="1">
+      <c r="A198" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="B198" s="4" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" ht="15" customHeight="1">
+      <c r="A199" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="B199" s="4" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" ht="15" customHeight="1">
+      <c r="A200" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="B200" s="4" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" ht="15" customHeight="1">
+      <c r="A201" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="B201" s="4" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" ht="15" customHeight="1">
+      <c r="A202" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="B202" s="4" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" ht="15" customHeight="1">
+      <c r="A203" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="B203" s="4" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" ht="15" customHeight="1">
+      <c r="A204" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="B204" s="4" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" ht="15" customHeight="1">
+      <c r="A205" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="B205" s="4" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" ht="15" customHeight="1">
+      <c r="A206" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="B206" s="4" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" ht="15" customHeight="1">
+      <c r="A207" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="B207" s="4" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" ht="15" customHeight="1">
+      <c r="A208" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="B208" s="4" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" ht="15" customHeight="1">
+      <c r="A209" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="B209" s="4" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" ht="15" customHeight="1">
+      <c r="A210" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="B210" s="4" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" ht="15" customHeight="1">
+      <c r="A211" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="B211" s="4" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" ht="15" customHeight="1">
+      <c r="A212" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="B212" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" ht="15" customHeight="1">
+      <c r="A213" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="B213" s="4" t="s">
+        <v>466</v>
       </c>
     </row>
   </sheetData>
@@ -6142,58 +6628,58 @@
     </row>
     <row r="89" spans="1:2" ht="15" customHeight="1">
       <c r="A89" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="15" customHeight="1">
       <c r="A90" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="15" customHeight="1">
       <c r="A91" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="15" customHeight="1">
       <c r="A92" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="15" customHeight="1">
       <c r="A93" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="15" customHeight="1">
       <c r="A94" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="15" customHeight="1">
       <c r="A95" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="15" customHeight="1">
@@ -6206,682 +6692,682 @@
     </row>
     <row r="97" spans="1:2" ht="15" customHeight="1">
       <c r="A97" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="15" customHeight="1">
       <c r="A98" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="15" customHeight="1">
       <c r="A99" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="15" customHeight="1">
       <c r="A100" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="15" customHeight="1">
       <c r="A101" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="15" customHeight="1">
       <c r="A102" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="15" customHeight="1">
       <c r="A103" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="15" customHeight="1">
       <c r="A104" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="105" spans="1:2" ht="15" customHeight="1">
       <c r="A105" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="15" customHeight="1">
       <c r="A106" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="15" customHeight="1">
       <c r="A107" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="15" customHeight="1">
       <c r="A108" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="15" customHeight="1">
       <c r="A109" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="110" spans="1:2" ht="15" customHeight="1">
       <c r="A110" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="15" customHeight="1">
       <c r="A111" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="15" customHeight="1">
       <c r="A112" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="113" spans="1:2" ht="15" customHeight="1">
       <c r="A113" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="15" customHeight="1">
       <c r="A114" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="15" customHeight="1">
       <c r="A115" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="15" customHeight="1">
       <c r="A116" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="15" customHeight="1">
       <c r="A117" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="15" customHeight="1">
       <c r="A118" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="15" customHeight="1">
       <c r="A119" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="120" spans="1:2" ht="15" customHeight="1">
       <c r="A120" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="15" customHeight="1">
       <c r="A121" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="15" customHeight="1">
       <c r="A122" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="15" customHeight="1">
       <c r="A123" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="15" customHeight="1">
       <c r="A124" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="125" spans="1:2" ht="15" customHeight="1">
       <c r="A125" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="126" spans="1:2" ht="15" customHeight="1">
       <c r="A126" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="15" customHeight="1">
       <c r="A127" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="15" customHeight="1">
       <c r="A128" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="15" customHeight="1">
       <c r="A129" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="15" customHeight="1">
       <c r="A130" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="15" customHeight="1">
       <c r="A131" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="15" customHeight="1">
       <c r="A132" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="15" customHeight="1">
       <c r="A133" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="15" customHeight="1">
       <c r="A134" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="15" customHeight="1">
       <c r="A135" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="15" customHeight="1">
       <c r="A136" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="137" spans="1:2" ht="15" customHeight="1">
       <c r="A137" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="15" customHeight="1">
       <c r="A138" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="15" customHeight="1">
       <c r="A139" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="15" customHeight="1">
       <c r="A140" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="15" customHeight="1">
       <c r="A141" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="15" customHeight="1">
       <c r="A142" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="15" customHeight="1">
       <c r="A143" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="15" customHeight="1">
       <c r="A144" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="15" customHeight="1">
       <c r="A145" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B145" s="4" t="s">
         <v>272</v>
-      </c>
-      <c r="B145" s="4" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="15" customHeight="1">
       <c r="A146" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B146" s="4" t="s">
         <v>274</v>
-      </c>
-      <c r="B146" s="4" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="15" customHeight="1">
       <c r="A147" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B147" s="4" t="s">
         <v>276</v>
-      </c>
-      <c r="B147" s="4" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="15" customHeight="1">
       <c r="A148" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B148" s="4" t="s">
         <v>278</v>
-      </c>
-      <c r="B148" s="4" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="15" customHeight="1">
       <c r="A149" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B149" s="4" t="s">
         <v>280</v>
-      </c>
-      <c r="B149" s="4" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="15" customHeight="1">
       <c r="A150" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B150" s="4" t="s">
         <v>282</v>
-      </c>
-      <c r="B150" s="4" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="15" customHeight="1">
       <c r="A151" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B151" s="4" t="s">
         <v>284</v>
-      </c>
-      <c r="B151" s="4" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="15" customHeight="1">
       <c r="A152" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B152" s="4" t="s">
         <v>286</v>
-      </c>
-      <c r="B152" s="4" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="15" customHeight="1">
       <c r="A153" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B153" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="15" customHeight="1">
       <c r="A154" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B154" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="15" customHeight="1">
       <c r="A155" s="7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B155" s="7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="15" customHeight="1">
       <c r="A156" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B156" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="157" spans="1:2" ht="15" customHeight="1">
       <c r="A157" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B157" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="15" customHeight="1">
       <c r="A158" s="7" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B158" s="7" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="15" customHeight="1">
       <c r="A159" s="7" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B159" s="7" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="160" spans="1:2" ht="15" customHeight="1">
       <c r="A160" s="7" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B160" s="7" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="161" spans="1:2" ht="15" customHeight="1">
       <c r="A161" s="7" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B161" s="7" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="162" spans="1:2" ht="15" customHeight="1">
       <c r="A162" s="7" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B162" s="7" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="15" customHeight="1">
       <c r="A163" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="164" spans="1:2" ht="15" customHeight="1">
       <c r="A164" s="7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B164" s="7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="165" spans="1:2" ht="15" customHeight="1">
       <c r="A165" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B165" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="15" customHeight="1">
       <c r="A166" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B166" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="15" customHeight="1">
       <c r="A167" s="7" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B167" s="7" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="168" spans="1:2" ht="15" customHeight="1">
       <c r="A168" s="7" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B168" s="7" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="15" customHeight="1">
       <c r="A169" s="7" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B169" s="7" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="15" customHeight="1">
       <c r="A170" s="7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B170" s="7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="15" customHeight="1">
       <c r="A171" s="7" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B171" s="7" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="15" customHeight="1">
       <c r="A172" s="4" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="15" customHeight="1">
       <c r="A173" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B173" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="174" spans="1:2" ht="15" customHeight="1">
       <c r="A174" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B174" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="15" customHeight="1">
       <c r="A175" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B175" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="15" customHeight="1">
       <c r="A176" s="7" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B176" s="7" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="15" customHeight="1">
       <c r="A177" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B177" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="15" customHeight="1">
       <c r="A178" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B178" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="179" spans="1:2" ht="15" customHeight="1">
       <c r="A179" s="7" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B179" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="15" customHeight="1">
       <c r="A180" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B180" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="181" spans="1:2" ht="15" customHeight="1">
       <c r="A181" s="7" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B181" s="7" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding Français and Español as language options
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -8,21 +8,36 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF280B9-7165-46BC-883D-757AF7A03BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36070FD1-5192-4F52-ADEA-6E73AAF54B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
     <sheet name="Deutsch" sheetId="2" r:id="rId2"/>
-    <sheet name="English" sheetId="3" r:id="rId3"/>
+    <sheet name="Français" sheetId="4" r:id="rId3"/>
+    <sheet name="Español" sheetId="5" r:id="rId4"/>
+    <sheet name="English" sheetId="3" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1166" uniqueCount="494">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2066" uniqueCount="882">
   <si>
     <t>exiobase</t>
   </si>
@@ -1521,6 +1536,1170 @@
   </si>
   <si>
     <t>Mindestanteil</t>
+  </si>
+  <si>
+    <t>Análisis de la cadena de suministro</t>
+  </si>
+  <si>
+    <t>Unidad</t>
+  </si>
+  <si>
+    <t>Producción de bienes de consumo</t>
+  </si>
+  <si>
+    <t>Proveedores directos</t>
+  </si>
+  <si>
+    <t>Producción de insumos</t>
+  </si>
+  <si>
+    <t>Extracción de materias primas</t>
+  </si>
+  <si>
+    <t>Proveedores</t>
+  </si>
+  <si>
+    <t>Mundo</t>
+  </si>
+  <si>
+    <t>de</t>
+  </si>
+  <si>
+    <t>Selección</t>
+  </si>
+  <si>
+    <t>Visualización</t>
+  </si>
+  <si>
+    <t>Ajustes</t>
+  </si>
+  <si>
+    <t>Ajustes básicos</t>
+  </si>
+  <si>
+    <t>Idioma</t>
+  </si>
+  <si>
+    <t>Año</t>
+  </si>
+  <si>
+    <t>Mostrar índices</t>
+  </si>
+  <si>
+    <t>Selección de región</t>
+  </si>
+  <si>
+    <t>Borrar</t>
+  </si>
+  <si>
+    <t>Seleccionar todas las regiones</t>
+  </si>
+  <si>
+    <t>Selección de sector</t>
+  </si>
+  <si>
+    <t>Seleccionar todos los sectores</t>
+  </si>
+  <si>
+    <t>Resumen de la selección</t>
+  </si>
+  <si>
+    <t>No se ha seleccionado nada</t>
+  </si>
+  <si>
+    <t>Aplicar la selección actual</t>
+  </si>
+  <si>
+    <t>Restablecer todo</t>
+  </si>
+  <si>
+    <t>Regiones</t>
+  </si>
+  <si>
+    <t>Sectores</t>
+  </si>
+  <si>
+    <t>No hay regiones seleccionadas</t>
+  </si>
+  <si>
+    <t>No hay sectores seleccionados</t>
+  </si>
+  <si>
+    <t>Todas las regiones seleccionadas (vista global)</t>
+  </si>
+  <si>
+    <t>Todos los sectores seleccionados (vista global)</t>
+  </si>
+  <si>
+    <t>Número de regiones</t>
+  </si>
+  <si>
+    <t>Número de sectores</t>
+  </si>
+  <si>
+    <t>Mapa mundial</t>
+  </si>
+  <si>
+    <t>Seleccionar indicadores ambientales</t>
+  </si>
+  <si>
+    <t>Seleccionado</t>
+  </si>
+  <si>
+    <t>Actualizar gráfico</t>
+  </si>
+  <si>
+    <t>Restablecer</t>
+  </si>
+  <si>
+    <t>una</t>
+  </si>
+  <si>
+    <t>selección específica de sectores</t>
+  </si>
+  <si>
+    <t>Por favor, selecciona primero sectores y regiones</t>
+  </si>
+  <si>
+    <t>Opciones</t>
+  </si>
+  <si>
+    <t>Consola</t>
+  </si>
+  <si>
+    <t>Consola interactiva</t>
+  </si>
+  <si>
+    <t>Ejecutar</t>
+  </si>
+  <si>
+    <t>se necesita más entrada</t>
+  </si>
+  <si>
+    <t>Actualizar mapa mundial</t>
+  </si>
+  <si>
+    <t>Por favor, actualiza</t>
+  </si>
+  <si>
+    <t>del mundo</t>
+  </si>
+  <si>
+    <t>Gráfico</t>
+  </si>
+  <si>
+    <t>Guardar gráfico</t>
+  </si>
+  <si>
+    <t>Archivo PNG (*.png)</t>
+  </si>
+  <si>
+    <t>Proporción global</t>
+  </si>
+  <si>
+    <t>Región</t>
+  </si>
+  <si>
+    <t>Información</t>
+  </si>
+  <si>
+    <t>Introduce el código Python abajo. Pulsa la tecla &lt;b&gt;Enter&lt;/b&gt; para ejecutarlo y usa &lt;b&gt;Mayús+Enter&lt;/b&gt; para insertar una nueva línea dentro de una instrucción de varias líneas.</t>
+  </si>
+  <si>
+    <t>Borrar salida</t>
+  </si>
+  <si>
+    <t>Salida de la consola</t>
+  </si>
+  <si>
+    <t>Apariencia</t>
+  </si>
+  <si>
+    <t>Preferencia del sistema</t>
+  </si>
+  <si>
+    <t>Modo claro</t>
+  </si>
+  <si>
+    <t>Modo oscuro</t>
+  </si>
+  <si>
+    <t>Color del mapa</t>
+  </si>
+  <si>
+    <t>Mostrar leyenda</t>
+  </si>
+  <si>
+    <t>Título (opcional)</t>
+  </si>
+  <si>
+    <t>Clasificación</t>
+  </si>
+  <si>
+    <t>Modo</t>
+  </si>
+  <si>
+    <t>continuo</t>
+  </si>
+  <si>
+    <t>por intervalos</t>
+  </si>
+  <si>
+    <t>Clases (k)</t>
+  </si>
+  <si>
+    <t>Clases personalizadas (separadas por comas)</t>
+  </si>
+  <si>
+    <t>Normalización (modo continuo)</t>
+  </si>
+  <si>
+    <t>Norma</t>
+  </si>
+  <si>
+    <t>lineal</t>
+  </si>
+  <si>
+    <t>logarítmica</t>
+  </si>
+  <si>
+    <t>intensa</t>
+  </si>
+  <si>
+    <t>Recorte robusto (%)</t>
+  </si>
+  <si>
+    <t>Gamma (norma de potencia)</t>
+  </si>
+  <si>
+    <t>Gráfico circular</t>
+  </si>
+  <si>
+    <t>Gráfico de burbujas</t>
+  </si>
+  <si>
+    <t>Diagrama de Sankey</t>
+  </si>
+  <si>
+    <t>Mapa de árbol (treemap)</t>
+  </si>
+  <si>
+    <t>Análisis por etapas de la cadena de valor</t>
+  </si>
+  <si>
+    <t>Análisis por regiones</t>
+  </si>
+  <si>
+    <t>Ajustes avanzados</t>
+  </si>
+  <si>
+    <t>Paleta de colores</t>
+  </si>
+  <si>
+    <t>Secuencial</t>
+  </si>
+  <si>
+    <t>Divergente</t>
+  </si>
+  <si>
+    <t>Cíclica</t>
+  </si>
+  <si>
+    <t>Cualitativa</t>
+  </si>
+  <si>
+    <t>Invertir</t>
+  </si>
+  <si>
+    <t>Tonos rojos</t>
+  </si>
+  <si>
+    <t>Tonos azules</t>
+  </si>
+  <si>
+    <t>Tonos verdes</t>
+  </si>
+  <si>
+    <t>Tonos violetas</t>
+  </si>
+  <si>
+    <t>Tonos naranjas</t>
+  </si>
+  <si>
+    <t>Tonos grises</t>
+  </si>
+  <si>
+    <t>Amarillo–Verde</t>
+  </si>
+  <si>
+    <t>Amarillo–Verde–Azul</t>
+  </si>
+  <si>
+    <t>Verde–Azul</t>
+  </si>
+  <si>
+    <t>Azul–Verde</t>
+  </si>
+  <si>
+    <t>Violeta–Azul</t>
+  </si>
+  <si>
+    <t>Azul–Violeta</t>
+  </si>
+  <si>
+    <t>Naranja–Rojo</t>
+  </si>
+  <si>
+    <t>Violeta–Rojo</t>
+  </si>
+  <si>
+    <t>Rojo–Violeta</t>
+  </si>
+  <si>
+    <t>Amarillo–Naranja–Marrón</t>
+  </si>
+  <si>
+    <t>Amarillo–Naranja–Rojo</t>
+  </si>
+  <si>
+    <t>Marrón–Verde azulado</t>
+  </si>
+  <si>
+    <t>Rosa–Amarillo verdoso</t>
+  </si>
+  <si>
+    <t>Púrpura–Verde</t>
+  </si>
+  <si>
+    <t>Violeta–Naranja</t>
+  </si>
+  <si>
+    <t>Rojo–Azul</t>
+  </si>
+  <si>
+    <t>Rojo–Gris</t>
+  </si>
+  <si>
+    <t>Rojo–Amarillo–Azul</t>
+  </si>
+  <si>
+    <t>Rojo–Amarillo–Verde</t>
+  </si>
+  <si>
+    <t>Espectral</t>
+  </si>
+  <si>
+    <t>Frío–Cálido</t>
+  </si>
+  <si>
+    <t>Azul–Blanco–Rojo</t>
+  </si>
+  <si>
+    <t>Sísmico</t>
+  </si>
+  <si>
+    <t>Crepúsculo (Twilight)</t>
+  </si>
+  <si>
+    <t>Crepúsculo (desplazado)</t>
+  </si>
+  <si>
+    <t>Acento</t>
+  </si>
+  <si>
+    <t>Oscuro 2</t>
+  </si>
+  <si>
+    <t>Otros</t>
+  </si>
+  <si>
+    <t>Porciones principales</t>
+  </si>
+  <si>
+    <t>Porcentaje mínimo (%)</t>
+  </si>
+  <si>
+    <t>Ordenar porciones</t>
+  </si>
+  <si>
+    <t>descendente</t>
+  </si>
+  <si>
+    <t>ascendente</t>
+  </si>
+  <si>
+    <t>en sentido antihorario</t>
+  </si>
+  <si>
+    <t>Ángulo inicial</t>
+  </si>
+  <si>
+    <t>Ajustes del gráfico circular</t>
+  </si>
+  <si>
+    <t>Límite excedido</t>
+  </si>
+  <si>
+    <t>Por favor, selecciona como máximo 3 impactos.</t>
+  </si>
+  <si>
+    <t>Seleccionar todo</t>
+  </si>
+  <si>
+    <t>Comparar con otros impactos</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
+    <t>Relativo (%)</t>
+  </si>
+  <si>
+    <t>Color de barras</t>
+  </si>
+  <si>
+    <t>Ancho de barras</t>
+  </si>
+  <si>
+    <t>Ajustes Top/Flop</t>
+  </si>
+  <si>
+    <t>Selecciona hasta 3 impactos para comparar.</t>
+  </si>
+  <si>
+    <t>Abrir ajustes</t>
+  </si>
+  <si>
+    <t>Actualizar</t>
+  </si>
+  <si>
+    <t>Exportar datos (Excel)</t>
+  </si>
+  <si>
+    <t>Impactos</t>
+  </si>
+  <si>
+    <t>Incluir unidades en los nombres de las columnas</t>
+  </si>
+  <si>
+    <t>Archivo de salida</t>
+  </si>
+  <si>
+    <t>Archivos de Excel (*.xlsx)</t>
+  </si>
+  <si>
+    <t>Selecciona al menos un impacto.</t>
+  </si>
+  <si>
+    <t>Por favor, elige un archivo .xlsx.</t>
+  </si>
+  <si>
+    <t>Exportación a Excel completada</t>
+  </si>
+  <si>
+    <t>Error al exportar a Excel</t>
+  </si>
+  <si>
+    <t>Seleccionar impactos</t>
+  </si>
+  <si>
+    <t>Continuo: los colores y la leyenda se basan en valores absolutos. Controla el contraste mediante normalización + recorte robusto + gamma.</t>
+  </si>
+  <si>
+    <t>Por intervalos: clases discretas. Con “Relativo”, clasificas por porcentajes (suma = 100 %); si no, por valores absolutos.</t>
+  </si>
+  <si>
+    <t>Representación</t>
+  </si>
+  <si>
+    <t>Definición de clases (por intervalos)</t>
+  </si>
+  <si>
+    <t>Relativo</t>
+  </si>
+  <si>
+    <t>Escala continua (continuo)</t>
+  </si>
+  <si>
+    <t>Normalización</t>
+  </si>
+  <si>
+    <t>Elige una paleta de colores para el mapa.</t>
+  </si>
+  <si>
+    <t>Invierte la paleta de colores.</t>
+  </si>
+  <si>
+    <t>Muestra la escala de colores con rangos de valores.</t>
+  </si>
+  <si>
+    <t>Título opcional encima del mapa.</t>
+  </si>
+  <si>
+    <t>Elige entre clases discretas (por intervalos) y escala continua (continuo).</t>
+  </si>
+  <si>
+    <t>Si está activo, las clases se forman por porcentajes (suma = 100 %); si no, por valores absolutos.</t>
+  </si>
+  <si>
+    <t>Número de clases si no se indican límites personalizados.</t>
+  </si>
+  <si>
+    <t>Límites internos de clase separados por comas. Mínimo y máximo se añaden automáticamente.</t>
+  </si>
+  <si>
+    <t>lineal: pasos uniformes | log: resalta órdenes de magnitud (logarítmico) | potencia: contraste ajustable con gamma</t>
+  </si>
+  <si>
+    <t>Determina vmin/vmax mediante cuantiles (p. ej., 2 % usa el percentil 2 y el 98).</t>
+  </si>
+  <si>
+    <t>Exponente para PowerNorm: &lt;1 resalta valores pequeños, &gt;1 resalta valores grandes.</t>
+  </si>
+  <si>
+    <t>Paleta de colores para colorear los países. Con “Invertir” se invierte el orden claro/oscuro.</t>
+  </si>
+  <si>
+    <t>Invierte la paleta seleccionada.</t>
+  </si>
+  <si>
+    <t>Muestra una leyenda. En modo “continuo” muestra valores absolutos; en modo “por intervalos” muestra rangos numéricos de clase.</t>
+  </si>
+  <si>
+    <t>Título opcional para el mapa.</t>
+  </si>
+  <si>
+    <t>continuo: los colores reflejan valores absolutos; la leyenda es continua. por intervalos: clases discretas. Con “Relativo” la división se hace por porcentajes.</t>
+  </si>
+  <si>
+    <t>Solo en modo por intervalos: alterna entre valores absolutos y porcentajes para los límites de clase.</t>
+  </si>
+  <si>
+    <t>Número de clases discretas. Si hay “Clases personalizadas”, estas tienen prioridad.</t>
+  </si>
+  <si>
+    <t>Introduce bordes internos, p. ej. “10, 25, 50”. Mínimo y máximo se añaden automáticamente.</t>
+  </si>
+  <si>
+    <t>Normalización para el modo continuo: - lineal: mapeo uniforme de vmin..vmax - log: mapeo logarítmico; solo para valores estrictamente positivos - potencia: mapeo por potencia; ver Gamma</t>
+  </si>
+  <si>
+    <t>El recorte robusto determina vmin/vmax por cuantiles en lugar de min/máx para amortiguar valores atípicos.</t>
+  </si>
+  <si>
+    <t>Gamma (PowerNorm): - gamma &lt; 1 resalta la parte baja - gamma &gt; 1 resalta la parte alta</t>
+  </si>
+  <si>
+    <t>Lineal: gradación uniforme de color de vmin a vmax.</t>
+  </si>
+  <si>
+    <t>Log: resalta órdenes de magnitud; requiere datos estrictamente positivos.</t>
+  </si>
+  <si>
+    <t>Potencia: controla el contraste con gamma (&lt;1: resalta valores pequeños; &gt;1: resalta valores grandes).</t>
+  </si>
+  <si>
+    <t>Ayuda</t>
+  </si>
+  <si>
+    <t>per cápita</t>
+  </si>
+  <si>
+    <t>Datos</t>
+  </si>
+  <si>
+    <t>El primer impacto determina el orden. Con el botón “Comparar con otros impactos” se pueden añadir hasta tres impactos para comparación.</t>
+  </si>
+  <si>
+    <t>Usar umbral de porcentaje mínimo</t>
+  </si>
+  <si>
+    <t>Configura cómo se seleccionan, ordenan y muestran las porciones. Consejo: si se activa un porcentaje mínimo, se ignora el límite de “Porciones principales”.</t>
+  </si>
+  <si>
+    <t>Modo porciones principales: se muestran las porciones más grandes; el resto se agrupa en “Otros”.</t>
+  </si>
+  <si>
+    <t>Modo umbral: las porciones por debajo del porcentaje mínimo se agrupan en “Otros”.</t>
+  </si>
+  <si>
+    <t>orden original</t>
+  </si>
+  <si>
+    <t>ascendente (más pequeñas primero)</t>
+  </si>
+  <si>
+    <t>descendente (más grandes primero)</t>
+  </si>
+  <si>
+    <t>Porcentaje mínimo</t>
+  </si>
+  <si>
+    <t>Analyse de la chaîne d’approvisionnement</t>
+  </si>
+  <si>
+    <t>Unité</t>
+  </si>
+  <si>
+    <t>Couleur</t>
+  </si>
+  <si>
+    <t>Production de biens de consommation</t>
+  </si>
+  <si>
+    <t>Fournisseurs directs</t>
+  </si>
+  <si>
+    <t>Production d’intrants</t>
+  </si>
+  <si>
+    <t>Extraction de matières premières</t>
+  </si>
+  <si>
+    <t>Fournisseurs</t>
+  </si>
+  <si>
+    <t>Monde</t>
+  </si>
+  <si>
+    <t>Sélection</t>
+  </si>
+  <si>
+    <t>Paramètres</t>
+  </si>
+  <si>
+    <t>Langue</t>
+  </si>
+  <si>
+    <t>Année</t>
+  </si>
+  <si>
+    <t>Afficher les indices</t>
+  </si>
+  <si>
+    <t>Effacer</t>
+  </si>
+  <si>
+    <t>Sélectionner toutes les régions</t>
+  </si>
+  <si>
+    <t>Sélectionner tous les secteurs</t>
+  </si>
+  <si>
+    <t>Appliquer la sélection actuelle</t>
+  </si>
+  <si>
+    <t>Régions</t>
+  </si>
+  <si>
+    <t>Secteurs</t>
+  </si>
+  <si>
+    <t>Aucune région sélectionnée</t>
+  </si>
+  <si>
+    <t>Aucun secteur sélectionné</t>
+  </si>
+  <si>
+    <t>Toutes les régions sélectionnées (vue globale)</t>
+  </si>
+  <si>
+    <t>Tous les secteurs sélectionnés (vue globale)</t>
+  </si>
+  <si>
+    <t>Nombre de régions</t>
+  </si>
+  <si>
+    <t>Nombre de secteurs</t>
+  </si>
+  <si>
+    <t>Carte du monde</t>
+  </si>
+  <si>
+    <t>Sélectionner des indicateurs environnementaux</t>
+  </si>
+  <si>
+    <t>Sélectionné</t>
+  </si>
+  <si>
+    <t>Réinitialiser</t>
+  </si>
+  <si>
+    <t>sélection spécifique de secteurs</t>
+  </si>
+  <si>
+    <t>Veuillez d’abord sélectionner des secteurs et des régions</t>
+  </si>
+  <si>
+    <t>Console interactive</t>
+  </si>
+  <si>
+    <t>Exécuter</t>
+  </si>
+  <si>
+    <t>Erreur</t>
+  </si>
+  <si>
+    <t>du monde</t>
+  </si>
+  <si>
+    <t>Graphique</t>
+  </si>
+  <si>
+    <t>Enregistrer le graphique</t>
+  </si>
+  <si>
+    <t>Fichier PNG (*.png)</t>
+  </si>
+  <si>
+    <t>Région</t>
+  </si>
+  <si>
+    <t>Effacer la sortie</t>
+  </si>
+  <si>
+    <t>Sortie de la console</t>
+  </si>
+  <si>
+    <t>Apparence</t>
+  </si>
+  <si>
+    <t>Mode clair</t>
+  </si>
+  <si>
+    <t>Mode sombre</t>
+  </si>
+  <si>
+    <t>Couleur de la carte</t>
+  </si>
+  <si>
+    <t>Afficher la légende</t>
+  </si>
+  <si>
+    <t>Titre (optionnel)</t>
+  </si>
+  <si>
+    <t>continu</t>
+  </si>
+  <si>
+    <t>Classes personnalisées (séparées par des virgules)</t>
+  </si>
+  <si>
+    <t>Normalisation (mode continu)</t>
+  </si>
+  <si>
+    <t>Norme</t>
+  </si>
+  <si>
+    <t>linéaire</t>
+  </si>
+  <si>
+    <t>logarithmique</t>
+  </si>
+  <si>
+    <t>Diagramme à bulles</t>
+  </si>
+  <si>
+    <t>Diagramme de Sankey</t>
+  </si>
+  <si>
+    <t>Analyse par régions</t>
+  </si>
+  <si>
+    <t>Paramètres avancés</t>
+  </si>
+  <si>
+    <t>Palette de couleurs</t>
+  </si>
+  <si>
+    <t>Perceptuelle</t>
+  </si>
+  <si>
+    <t>Séquentielle</t>
+  </si>
+  <si>
+    <t>Cyclique</t>
+  </si>
+  <si>
+    <t>Inverser</t>
+  </si>
+  <si>
+    <t>Tons rouges</t>
+  </si>
+  <si>
+    <t>Tons bleus</t>
+  </si>
+  <si>
+    <t>Tons verts</t>
+  </si>
+  <si>
+    <t>Tons violets</t>
+  </si>
+  <si>
+    <t>Tons gris</t>
+  </si>
+  <si>
+    <t>Jaune–Vert</t>
+  </si>
+  <si>
+    <t>Jaune–Vert–Bleu</t>
+  </si>
+  <si>
+    <t>Vert–Bleu</t>
+  </si>
+  <si>
+    <t>Bleu–Vert</t>
+  </si>
+  <si>
+    <t>Violet–Bleu</t>
+  </si>
+  <si>
+    <t>Bleu–Violet</t>
+  </si>
+  <si>
+    <t>Orange–Rouge</t>
+  </si>
+  <si>
+    <t>Violet–Rouge</t>
+  </si>
+  <si>
+    <t>Rouge–Violet</t>
+  </si>
+  <si>
+    <t>Jaune–Orange–Brun</t>
+  </si>
+  <si>
+    <t>Jaune–Orange–Rouge</t>
+  </si>
+  <si>
+    <t>Brun–Bleu-vert</t>
+  </si>
+  <si>
+    <t>Rose–Jaune-vert</t>
+  </si>
+  <si>
+    <t>Pourpre–Vert</t>
+  </si>
+  <si>
+    <t>Violet–Orange</t>
+  </si>
+  <si>
+    <t>Rouge–Bleu</t>
+  </si>
+  <si>
+    <t>Rouge–Gris</t>
+  </si>
+  <si>
+    <t>Rouge–Jaune–Bleu</t>
+  </si>
+  <si>
+    <t>Rouge–Jaune–Vert</t>
+  </si>
+  <si>
+    <t>Froid–Chaud</t>
+  </si>
+  <si>
+    <t>Bleu–Blanc–Rouge</t>
+  </si>
+  <si>
+    <t>Sismique</t>
+  </si>
+  <si>
+    <t>Twilight (décalé)</t>
+  </si>
+  <si>
+    <t>Autres</t>
+  </si>
+  <si>
+    <t>Tranches principales</t>
+  </si>
+  <si>
+    <t>Part minimale (%)</t>
+  </si>
+  <si>
+    <t>Trier les tranches</t>
+  </si>
+  <si>
+    <t>décroissant</t>
+  </si>
+  <si>
+    <t>croissant</t>
+  </si>
+  <si>
+    <t>Angle de départ</t>
+  </si>
+  <si>
+    <t>Limite dépassée</t>
+  </si>
+  <si>
+    <t>Veuillez sélectionner au maximum 3 impacts.</t>
+  </si>
+  <si>
+    <t>Tout sélectionner</t>
+  </si>
+  <si>
+    <t>Comparer avec d’autres impacts</t>
+  </si>
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>Relatif (%)</t>
+  </si>
+  <si>
+    <t>Couleur des barres</t>
+  </si>
+  <si>
+    <t>Largeur des barres</t>
+  </si>
+  <si>
+    <t>Paramètres Top/Flop</t>
+  </si>
+  <si>
+    <t>Sélectionnez jusqu’à 3 impacts à comparer.</t>
+  </si>
+  <si>
+    <t>Ouvrir les paramètres</t>
+  </si>
+  <si>
+    <t>Exporter les données (Excel)</t>
+  </si>
+  <si>
+    <t>Inclure les unités dans les noms de colonnes</t>
+  </si>
+  <si>
+    <t>Fichier de sortie</t>
+  </si>
+  <si>
+    <t>Fichiers Excel (*.xlsx)</t>
+  </si>
+  <si>
+    <t>Veuillez sélectionner au moins un impact.</t>
+  </si>
+  <si>
+    <t>Veuillez choisir un fichier .xlsx.</t>
+  </si>
+  <si>
+    <t>Export Excel terminé</t>
+  </si>
+  <si>
+    <t>Erreur lors de l’export Excel</t>
+  </si>
+  <si>
+    <t>Sélectionner des impacts</t>
+  </si>
+  <si>
+    <t>Relatif</t>
+  </si>
+  <si>
+    <t>Normalisation</t>
+  </si>
+  <si>
+    <t>Choisissez une palette de couleurs pour la carte.</t>
+  </si>
+  <si>
+    <t>Inverse la palette de couleurs.</t>
+  </si>
+  <si>
+    <t>Titre optionnel au-dessus de la carte.</t>
+  </si>
+  <si>
+    <t>Si activé, les classes sont formées selon des parts en pourcentage (somme = 100 %) ; sinon selon des valeurs absolues.</t>
+  </si>
+  <si>
+    <t>Détermine vmin/vmax via des quantiles (p. ex. 2 % utilise les 2e et 98e percentiles).</t>
+  </si>
+  <si>
+    <t>Titre optionnel pour la carte.</t>
+  </si>
+  <si>
+    <t>Aide</t>
+  </si>
+  <si>
+    <t>par habitant</t>
+  </si>
+  <si>
+    <t>Données</t>
+  </si>
+  <si>
+    <t>Utiliser un seuil de part minimale</t>
+  </si>
+  <si>
+    <t>Paramètres de base</t>
+  </si>
+  <si>
+    <t>Sélection de région</t>
+  </si>
+  <si>
+    <t>Sélection de secteur</t>
+  </si>
+  <si>
+    <t>Résumé de la sélection</t>
+  </si>
+  <si>
+    <t>Aucune sélection</t>
+  </si>
+  <si>
+    <t>Tout réinitialiser</t>
+  </si>
+  <si>
+    <t>Mettre à jour le graphique</t>
+  </si>
+  <si>
+    <t>une</t>
+  </si>
+  <si>
+    <t>plus de saisie requise</t>
+  </si>
+  <si>
+    <t>Mettre à jour la carte du monde</t>
+  </si>
+  <si>
+    <t>Veuillez mettre à jour</t>
+  </si>
+  <si>
+    <t>Part globale</t>
+  </si>
+  <si>
+    <t>Informations</t>
+  </si>
+  <si>
+    <t>Saisissez le code Python ci-dessous. Appuyez sur la touche &lt;b&gt;Entrée&lt;/b&gt; pour l’exécuter et utilisez &lt;b&gt;Maj+Entrée&lt;/b&gt; pour insérer une nouvelle ligne dans une instruction sur plusieurs lignes.</t>
+  </si>
+  <si>
+    <t>Préférence du système</t>
+  </si>
+  <si>
+    <t>par classes</t>
+  </si>
+  <si>
+    <t>intense</t>
+  </si>
+  <si>
+    <t>Troncature robuste (%)</t>
+  </si>
+  <si>
+    <t>Gamma (norme puissance)</t>
+  </si>
+  <si>
+    <t>Diagramme circulaire</t>
+  </si>
+  <si>
+    <t>Treemap (carte arborescente)</t>
+  </si>
+  <si>
+    <t>Analyse par niveaux de la chaîne de valeur</t>
+  </si>
+  <si>
+    <t>Tons orange</t>
+  </si>
+  <si>
+    <t>Dark 2</t>
+  </si>
+  <si>
+    <t>dans le sens antihoraire</t>
+  </si>
+  <si>
+    <t>Paramètres du diagramme circulaire</t>
+  </si>
+  <si>
+    <t>Mettre à jour</t>
+  </si>
+  <si>
+    <t>Continu : couleurs et légende basées sur des valeurs absolues. Le contraste se règle via normalisation + troncature robuste + gamma.</t>
+  </si>
+  <si>
+    <t>Par classes : classes discrètes. Avec « Relatif », la classification se fait par pourcentages (somme = 100 %) ; sinon, par valeurs absolues.</t>
+  </si>
+  <si>
+    <t>Représentation</t>
+  </si>
+  <si>
+    <t>Découpage en classes (par classes)</t>
+  </si>
+  <si>
+    <t>Échelle continue (continu)</t>
+  </si>
+  <si>
+    <t>Affiche l’échelle de couleurs avec des plages de valeurs.</t>
+  </si>
+  <si>
+    <t>Choisissez entre classes discrètes (par classes) et échelle continue (continu).</t>
+  </si>
+  <si>
+    <t>Nombre de classes si aucun seuil personnalisé n’est indiqué.</t>
+  </si>
+  <si>
+    <t>Seuils internes des classes séparés par des virgules. Le minimum et le maximum sont ajoutés automatiquement.</t>
+  </si>
+  <si>
+    <t>linéaire : pas réguliers | log : met l’accent sur les ordres de grandeur (logarithmique) | puissance : contraste ajustable avec gamma</t>
+  </si>
+  <si>
+    <t>Exposant pour PowerNorm : &lt;1 met en avant les petites valeurs, &gt;1 met en avant les grandes valeurs.</t>
+  </si>
+  <si>
+    <t>Palette pour colorer les pays. Avec « Inverser », l’ordre clair/foncé est inversé.</t>
+  </si>
+  <si>
+    <t>Inverse la palette choisie.</t>
+  </si>
+  <si>
+    <t>Affiche une légende. En mode « continu », elle montre des valeurs absolues ; en mode « par classes », elle montre des plages numériques de classes.</t>
+  </si>
+  <si>
+    <t>continu : les couleurs reflètent des valeurs absolues ; la légende est continue. par classes : classes discrètes. Avec « Relatif », le découpage se fait par pourcentages.</t>
+  </si>
+  <si>
+    <t>Uniquement en mode par classes : bascule entre valeurs absolues et pourcentages pour les seuils de classes.</t>
+  </si>
+  <si>
+    <t>Nombre de classes discrètes. Si « Classes personnalisées » est renseigné, celles-ci priment.</t>
+  </si>
+  <si>
+    <t>Saisissez des seuils internes, p. ex. « 10, 25, 50 ». Le minimum et le maximum sont ajoutés automatiquement.</t>
+  </si>
+  <si>
+    <t>Normalisation pour le mode continu : - linéaire : mappage uniforme de vmin..vmax - log : mappage logarithmique ; uniquement pour des valeurs strictement positives - puissance : mappage en puissance ; voir Gamma</t>
+  </si>
+  <si>
+    <t>La troncature robuste détermine vmin/vmax via des quantiles plutôt que via min/max afin d’atténuer les valeurs aberrantes.</t>
+  </si>
+  <si>
+    <t>Gamma (PowerNorm) : - gamma &lt; 1 met en avant la partie basse - gamma &gt; 1 met en avant la partie haute</t>
+  </si>
+  <si>
+    <t>Linéaire : dégradé de couleurs régulier de vmin à vmax.</t>
+  </si>
+  <si>
+    <t>Log : met l’accent sur les ordres de grandeur ; nécessite des données strictement positives.</t>
+  </si>
+  <si>
+    <t>Puissance : contrôle du contraste via gamma (&lt;1 : met en avant les petites valeurs ; &gt;1 : met en avant les grandes).</t>
+  </si>
+  <si>
+    <t>Le premier impact détermine l’ordre. Via le bouton « Comparer avec d’autres impacts », on peut ajouter jusqu’à trois impacts de comparaison.</t>
+  </si>
+  <si>
+    <t>Configurez comment les tranches sont sélectionnées, triées et affichées. Astuce : si une part minimale est activée, la limite « Tranches principales » est ignorée.</t>
+  </si>
+  <si>
+    <t>Mode tranches principales : les plus grandes tranches sont affichées, le reste est regroupé sous « Autres ».</t>
+  </si>
+  <si>
+    <t>Mode seuil : les parts en dessous de la part minimale sont regroupées sous « Autres ».</t>
+  </si>
+  <si>
+    <t>ordre d’origine</t>
+  </si>
+  <si>
+    <t>croissant (les plus petites d’abord)</t>
+  </si>
+  <si>
+    <t>décroissant (les plus grandes d’abord)</t>
+  </si>
+  <si>
+    <t>Part minimale</t>
   </si>
 </sst>
 </file>
@@ -6077,6 +7256,3634 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDF42DCD-97DE-4ED1-A72F-019B4378FB2B}">
+  <dimension ref="A1:B225"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="46.28515625" customWidth="1"/>
+    <col min="2" max="2" width="196.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B37" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B38" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B44" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B46" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B51" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B52" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B54" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B55" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B56" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B57" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B58" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B59" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B60" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B61" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B62" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B63" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B64" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B65" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B66" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B67" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B68" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B69" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B70" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B71" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B72" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B73" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B74" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B75" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B76" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B77" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B78" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B79" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B80" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B81" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B83" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B84" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B85" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B86" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B87" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B88" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B89" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B90" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B91" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B92" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B93" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B94" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B95" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B96" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B97" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B98" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B99" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B100" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B101" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B102" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B103" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B104" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B105" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B106" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B107" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B108" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B109" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B110" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B111" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B112" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2">
+      <c r="A113" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B113" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B114" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B115" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B116" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B117" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B118" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B119" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B120" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B121" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B122" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B123" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B124" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B125" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B126" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B127" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B128" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B129" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="A130" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B130" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B131" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="B132" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B133" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="B134" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B135" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B136" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B137" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="B138" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B139" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B140" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B141" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B142" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B143" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B144" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B145" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B146" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B147" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B148" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="B149" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B150" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="B151" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="B152" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="B153" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="B154" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="B155" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="B156" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="B157" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="B158" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="B159" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B160" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="B161" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B162" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="B163" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="B164" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="B165" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="B166" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="B167" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="B168" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="B169" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="B170" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="B171" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="B172" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="B173" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="B174" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="B175" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="B176" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="B177" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="B178" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="B179" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="B180" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="B181" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="B182" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="B183" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="B184" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="B185" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="B186" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B187" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="B188" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="B189" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="B190" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="B191" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="B192" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="B193" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="B194" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="B195" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="B196" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="B197" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="B198" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="B199" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="B200" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="B201" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="B202" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2">
+      <c r="A203" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="B203" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2">
+      <c r="A204" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="B204" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2">
+      <c r="A205" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="B205" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2">
+      <c r="A206" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="B206" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2">
+      <c r="A207" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="B207" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2">
+      <c r="A208" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="B208" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
+      <c r="A209" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="B209" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
+      <c r="A210" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="B210" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
+      <c r="A211" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="B211" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="B212" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="A213" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="B213" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="B214" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="B215" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="B216" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="B217" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="B218" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="B219" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="B220" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="B221" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="B222" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="B223" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="B224" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="B225" t="s">
+        <v>881</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50CB9232-502D-4CCC-9B6B-AA584BDCDD9C}">
+  <dimension ref="A1:B225"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="47.7109375" customWidth="1"/>
+    <col min="2" max="2" width="127.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B65" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B92" s="7" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2">
+      <c r="A113" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="A130" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="B149" s="7" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B150" s="7" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="B151" s="7" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="B152" s="7" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="B153" s="7" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="B154" s="7" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="B155" s="7" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="B156" s="7" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="B157" s="7" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="B158" s="7" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="B159" s="7" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B160" s="7" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="B161" s="7" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B162" s="7" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="B163" s="7" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="B164" s="7" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="B165" s="7" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="B166" s="7" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="B167" s="7" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="B168" s="7" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="B170" s="7" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="B171" s="7" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="B172" s="7" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="B173" s="4" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="B174" s="4" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="B175" s="4" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="B176" s="7" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="B177" s="4" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="B178" s="4" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="B179" s="4" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="B180" s="7" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="B181" s="4" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="B182" s="4" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="B183" s="4" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="B184" s="4" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="B185" s="7" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="B186" s="4" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B187" s="4" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="B188" s="4" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="B189" s="4" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="B190" s="4" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="B191" s="4" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="B192" s="4" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="B193" s="4" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="B194" s="4" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="B195" s="4" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="B196" s="4" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="B197" s="4" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="B198" s="4" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="B199" s="4" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="B200" s="4" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="B201" s="4" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="B202" s="4" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2">
+      <c r="A203" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="B203" s="4" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2">
+      <c r="A204" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="B204" s="4" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2">
+      <c r="A205" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="B205" s="4" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2">
+      <c r="A206" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="B206" s="4" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2">
+      <c r="A207" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="B207" s="4" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2">
+      <c r="A208" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="B208" s="4" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
+      <c r="A209" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="B209" s="4" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
+      <c r="A210" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="B210" s="4" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
+      <c r="A211" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="B211" s="4" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="B212" s="4" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="A213" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="B213" s="4" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="B214" s="4" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="B215" s="4" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="B216" s="4" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="B217" s="4" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="B218" s="4" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="B219" s="4" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="B220" s="4" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="B221" s="4" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="B222" s="7" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="B223" s="7" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="B224" s="7" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="B225" s="4" t="s">
+        <v>692</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B181"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>

</xml_diff>

<commit_message>
chore(ui): i18n for remaining control labels
</commit_message>
<xml_diff>
--- a/config/general.xlsx
+++ b/config/general.xlsx
@@ -1302,7 +1302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J259"/>
+  <dimension ref="A1:J263"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="60.5703125" customWidth="1" style="4" min="1" max="1"/>
@@ -4434,6 +4434,54 @@
       <c r="B259" t="inlineStr">
         <is>
           <t>Set year and language here. This affects selection and analyses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Collapse</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Collapse</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Expand</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Expand</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Search?</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Search?</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Gamma</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Gamma</t>
         </is>
       </c>
     </row>
@@ -4457,7 +4505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B303"/>
+  <dimension ref="A1:B307"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="67" customWidth="1" style="4" min="1" max="1"/>
@@ -8126,6 +8174,54 @@
       <c r="B303" t="inlineStr">
         <is>
           <t>Hier stellst du Jahr und Sprache ein. Das wirkt auf Auswahl und Analysen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Collapse</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Einklappen</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Expand</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Aufklappen</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Search?</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Suchen?</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Gamma</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Gamma</t>
         </is>
       </c>
     </row>
@@ -8149,7 +8245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B303"/>
+  <dimension ref="A1:B307"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="46.28515625" customWidth="1" style="1" min="1" max="1"/>
@@ -11805,6 +11901,54 @@
       <c r="B303" t="inlineStr">
         <is>
           <t>Set year and language here. This affects selection and analyses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Collapse</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>R?duire</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Expand</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>D?velopper</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Search?</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Rechercher?</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Gamma</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Gamma</t>
         </is>
       </c>
     </row>
@@ -11819,7 +11963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B303"/>
+  <dimension ref="A1:B307"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="47.7109375" customWidth="1" style="1" min="1" max="1"/>
@@ -15475,6 +15619,54 @@
       <c r="B303" t="inlineStr">
         <is>
           <t>Set year and language here. This affects selection and analyses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Collapse</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Contraer</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Expand</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Expandir</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Search?</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Buscar?</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Gamma</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Gamma</t>
         </is>
       </c>
     </row>
@@ -15489,7 +15681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B263"/>
+  <dimension ref="A1:B267"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="64" customWidth="1" style="4" min="1" max="1"/>
@@ -18661,6 +18853,54 @@
       <c r="B263" t="inlineStr">
         <is>
           <t>Set year and language here. This affects selection and analyses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Collapse</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Collapse</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Expand</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Expand</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Search?</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Search?</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Gamma</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Gamma</t>
         </is>
       </c>
     </row>

</xml_diff>